<commit_message>
Agrego dato PIB 2T26, comex y res fiscal ago26
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183DEE59-9929-4CDF-AC5A-294038B79C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBC8E71-BF5A-4238-900B-3014B1CBBE25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="225">
   <si>
     <t>Período</t>
   </si>
@@ -915,7 +915,7 @@
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1008,8 +1008,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Euro" xfId="10" xr:uid="{8CA0DC4E-5AAC-43A0-AC51-59D877AC41AF}"/>
@@ -3370,10 +3368,10 @@
         <v>84</v>
       </c>
       <c r="B2">
-        <v>599983.70014804997</v>
+        <v>660900.72934956325</v>
       </c>
       <c r="C2">
-        <v>2.481356123815659</v>
+        <v>1.9987560115406033</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3381,10 +3379,10 @@
         <v>85</v>
       </c>
       <c r="B3">
-        <v>38842.924521107714</v>
+        <v>97139.886663930403</v>
       </c>
       <c r="C3">
-        <v>18.138938518629178</v>
+        <v>6.9486384806836998</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3392,10 +3390,10 @@
         <v>86</v>
       </c>
       <c r="B4">
-        <v>1545.6270924291682</v>
+        <v>2719.9519172511359</v>
       </c>
       <c r="C4">
-        <v>27.45728282807076</v>
+        <v>44.652720343850461</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3403,10 +3401,10 @@
         <v>87</v>
       </c>
       <c r="B5">
-        <v>30755.076629366038</v>
+        <v>34220.002463165692</v>
       </c>
       <c r="C5">
-        <v>12.334190997099181</v>
+        <v>16.365238681536741</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3414,10 +3412,10 @@
         <v>88</v>
       </c>
       <c r="B6">
-        <v>112761.23165011391</v>
+        <v>106823.39062635107</v>
       </c>
       <c r="C6">
-        <v>-1.676454111061576</v>
+        <v>-2.1320163173545237</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3425,10 +3423,10 @@
         <v>89</v>
       </c>
       <c r="B7">
-        <v>12673.907286977306</v>
+        <v>13356.112303267913</v>
       </c>
       <c r="C7">
-        <v>-1.0509245571815207</v>
+        <v>5.0191905864735986</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3436,10 +3434,10 @@
         <v>90</v>
       </c>
       <c r="B8">
-        <v>19017.800104434555</v>
+        <v>18998.084115102614</v>
       </c>
       <c r="C8">
-        <v>2.5370815997647345</v>
+        <v>0.23511441641870245</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3447,10 +3445,10 @@
         <v>91</v>
       </c>
       <c r="B9">
-        <v>91872.245634525272</v>
+        <v>95230.33054254642</v>
       </c>
       <c r="C9">
-        <v>-0.29307255440298441</v>
+        <v>4.9735461799071956E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3458,10 +3456,10 @@
         <v>92</v>
       </c>
       <c r="B10">
-        <v>13022.400979766842</v>
+        <v>11163.567159514021</v>
       </c>
       <c r="C10">
-        <v>2.7902948421734797</v>
+        <v>1.6463203839668816</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3469,10 +3467,10 @@
         <v>93</v>
       </c>
       <c r="B11">
-        <v>55633.327772916178</v>
+        <v>57999.422558425314</v>
       </c>
       <c r="C11">
-        <v>2.2858102158443083</v>
+        <v>1.6196813114308428</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3480,10 +3478,10 @@
         <v>94</v>
       </c>
       <c r="B12">
-        <v>30381.126773097683</v>
+        <v>29279.508420721446</v>
       </c>
       <c r="C12">
-        <v>7.5048032104928053</v>
+        <v>4.8159177343507276</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3491,10 +3489,10 @@
         <v>95</v>
       </c>
       <c r="B13">
-        <v>85939.774708283672</v>
+        <v>85616.367821990279</v>
       </c>
       <c r="C13">
-        <v>0.89683919333798379</v>
+        <v>0.67920914109178554</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3502,10 +3500,10 @@
         <v>96</v>
       </c>
       <c r="B14">
-        <v>34900.492729780119</v>
+        <v>34280.6780469078</v>
       </c>
       <c r="C14">
-        <v>-1.3759391935735277</v>
+        <v>-1.4398890487727356</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -3513,10 +3511,10 @@
         <v>97</v>
       </c>
       <c r="B15">
-        <v>29912.893832996058</v>
+        <v>29393.914507255231</v>
       </c>
       <c r="C15">
-        <v>5.5946826390473881E-2</v>
+        <v>0.11667222623130691</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -3524,10 +3522,10 @@
         <v>98</v>
       </c>
       <c r="B16">
-        <v>23085.607234226565</v>
+        <v>26301.382534738379</v>
       </c>
       <c r="C16">
-        <v>0.46783601580868694</v>
+        <v>0.46514355653639594</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -3535,10 +3533,10 @@
         <v>99</v>
       </c>
       <c r="B17">
-        <v>15478.186568411322</v>
+        <v>14521.040025832417</v>
       </c>
       <c r="C17">
-        <v>0.6554599397215588</v>
+        <v>-0.9029928198407533</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -3546,10 +3544,10 @@
         <v>100</v>
       </c>
       <c r="B18">
-        <v>4161.0766296179845</v>
+        <v>3857.0896425632591</v>
       </c>
       <c r="C18">
-        <v>6.2795181172130343</v>
+        <v>0.86908699909673537</v>
       </c>
     </row>
   </sheetData>
@@ -6036,25 +6034,25 @@
       <c r="A2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="52">
+      <c r="B2" s="33">
         <v>33.5</v>
       </c>
-      <c r="C2" s="52">
+      <c r="C2" s="33">
         <v>33.700000000000003</v>
       </c>
-      <c r="D2" s="52">
+      <c r="D2" s="33">
         <v>33.1</v>
       </c>
-      <c r="E2" s="52">
+      <c r="E2" s="33">
         <v>37</v>
       </c>
-      <c r="F2" s="52">
+      <c r="F2" s="33">
         <v>34</v>
       </c>
-      <c r="G2" s="52">
+      <c r="G2" s="33">
         <v>33.4</v>
       </c>
-      <c r="H2" s="52">
+      <c r="H2" s="33">
         <v>31.6</v>
       </c>
     </row>
@@ -6062,25 +6060,25 @@
       <c r="A3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="53">
+      <c r="B3" s="34">
         <v>34.9</v>
       </c>
-      <c r="C3" s="53">
+      <c r="C3" s="34">
         <v>34.299999999999997</v>
       </c>
-      <c r="D3" s="53">
+      <c r="D3" s="34">
         <v>34.9</v>
       </c>
-      <c r="E3" s="53">
+      <c r="E3" s="34">
         <v>41.8</v>
       </c>
-      <c r="F3" s="53">
+      <c r="F3" s="34">
         <v>37.299999999999997</v>
       </c>
-      <c r="G3" s="53">
+      <c r="G3" s="34">
         <v>34.799999999999997</v>
       </c>
-      <c r="H3" s="53">
+      <c r="H3" s="34">
         <v>30</v>
       </c>
     </row>
@@ -6088,25 +6086,25 @@
       <c r="A4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="53">
+      <c r="B4" s="34">
         <v>22.6</v>
       </c>
-      <c r="C4" s="53">
+      <c r="C4" s="34">
         <v>23.1</v>
       </c>
-      <c r="D4" s="53">
+      <c r="D4" s="34">
         <v>21.9</v>
       </c>
-      <c r="E4" s="53">
+      <c r="E4" s="34">
         <v>22.2</v>
       </c>
-      <c r="F4" s="53">
+      <c r="F4" s="34">
         <v>22.6</v>
       </c>
-      <c r="G4" s="53">
+      <c r="G4" s="34">
         <v>22.6</v>
       </c>
-      <c r="H4" s="53">
+      <c r="H4" s="34">
         <v>24.4</v>
       </c>
     </row>
@@ -6114,25 +6112,25 @@
       <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="53">
+      <c r="B5" s="34">
         <v>11</v>
       </c>
-      <c r="C5" s="53">
+      <c r="C5" s="34">
         <v>10</v>
       </c>
-      <c r="D5" s="53">
+      <c r="D5" s="34">
         <v>11.3</v>
       </c>
-      <c r="E5" s="53">
+      <c r="E5" s="34">
         <v>12.2</v>
       </c>
-      <c r="F5" s="53">
+      <c r="F5" s="34">
         <v>11.8</v>
       </c>
-      <c r="G5" s="53">
+      <c r="G5" s="34">
         <v>15.7</v>
       </c>
-      <c r="H5" s="53">
+      <c r="H5" s="34">
         <v>13.1</v>
       </c>
     </row>
@@ -6140,25 +6138,25 @@
       <c r="A6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="53">
+      <c r="B6" s="34">
         <v>49.1</v>
       </c>
-      <c r="C6" s="53">
+      <c r="C6" s="34">
         <v>45.3</v>
       </c>
-      <c r="D6" s="53">
+      <c r="D6" s="34">
         <v>49.3</v>
       </c>
-      <c r="E6" s="53">
+      <c r="E6" s="34">
         <v>74.5</v>
       </c>
-      <c r="F6" s="53">
+      <c r="F6" s="34">
         <v>50.1</v>
       </c>
-      <c r="G6" s="53">
+      <c r="G6" s="34">
         <v>50.8</v>
       </c>
-      <c r="H6" s="53">
+      <c r="H6" s="34">
         <v>50.9</v>
       </c>
     </row>
@@ -6166,25 +6164,25 @@
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="53">
+      <c r="B7" s="34">
         <v>24.4</v>
       </c>
-      <c r="C7" s="53">
+      <c r="C7" s="34">
         <v>25.8</v>
       </c>
-      <c r="D7" s="53">
+      <c r="D7" s="34">
         <v>24.1</v>
       </c>
-      <c r="E7" s="53">
+      <c r="E7" s="34">
         <v>18.5</v>
       </c>
-      <c r="F7" s="53">
+      <c r="F7" s="34">
         <v>24</v>
       </c>
-      <c r="G7" s="53">
+      <c r="G7" s="34">
         <v>22.4</v>
       </c>
-      <c r="H7" s="53">
+      <c r="H7" s="34">
         <v>21.4</v>
       </c>
     </row>
@@ -6192,25 +6190,25 @@
       <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="53">
+      <c r="B8" s="34">
         <v>33.200000000000003</v>
       </c>
-      <c r="C8" s="53">
+      <c r="C8" s="34">
         <v>33.299999999999997</v>
       </c>
-      <c r="D8" s="53">
+      <c r="D8" s="34">
         <v>33.700000000000003</v>
       </c>
-      <c r="E8" s="53">
+      <c r="E8" s="34">
         <v>31</v>
       </c>
-      <c r="F8" s="53">
+      <c r="F8" s="34">
         <v>32.200000000000003</v>
       </c>
-      <c r="G8" s="53">
+      <c r="G8" s="34">
         <v>31.3</v>
       </c>
-      <c r="H8" s="53">
+      <c r="H8" s="34">
         <v>33.6</v>
       </c>
     </row>
@@ -6218,25 +6216,25 @@
       <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="53">
+      <c r="B9" s="34">
         <v>38.200000000000003</v>
       </c>
-      <c r="C9" s="53">
+      <c r="C9" s="34">
         <v>38.6</v>
       </c>
-      <c r="D9" s="53">
+      <c r="D9" s="34">
         <v>37.1</v>
       </c>
-      <c r="E9" s="53">
+      <c r="E9" s="34">
         <v>31.1</v>
       </c>
-      <c r="F9" s="53">
+      <c r="F9" s="34">
         <v>42</v>
       </c>
-      <c r="G9" s="53">
+      <c r="G9" s="34">
         <v>42.1</v>
       </c>
-      <c r="H9" s="53">
+      <c r="H9" s="34">
         <v>38.700000000000003</v>
       </c>
     </row>
@@ -6244,25 +6242,25 @@
       <c r="A10" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="53">
+      <c r="B10" s="34">
         <v>36.799999999999997</v>
       </c>
-      <c r="C10" s="53">
+      <c r="C10" s="34">
         <v>38.200000000000003</v>
       </c>
-      <c r="D10" s="53">
+      <c r="D10" s="34">
         <v>35.9</v>
       </c>
-      <c r="E10" s="53">
+      <c r="E10" s="34">
         <v>34</v>
       </c>
-      <c r="F10" s="53">
+      <c r="F10" s="34">
         <v>36.299999999999997</v>
       </c>
-      <c r="G10" s="53">
+      <c r="G10" s="34">
         <v>35.299999999999997</v>
       </c>
-      <c r="H10" s="53">
+      <c r="H10" s="34">
         <v>34.5</v>
       </c>
     </row>
@@ -6270,25 +6268,25 @@
       <c r="A11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="53">
+      <c r="B11" s="34">
         <v>31.5</v>
       </c>
-      <c r="C11" s="53">
+      <c r="C11" s="34">
         <v>33.200000000000003</v>
       </c>
-      <c r="D11" s="53">
+      <c r="D11" s="34">
         <v>31.5</v>
       </c>
-      <c r="E11" s="53">
+      <c r="E11" s="34">
         <v>28.8</v>
       </c>
-      <c r="F11" s="53">
+      <c r="F11" s="34">
         <v>28.5</v>
       </c>
-      <c r="G11" s="53">
+      <c r="G11" s="34">
         <v>28</v>
       </c>
-      <c r="H11" s="53">
+      <c r="H11" s="34">
         <v>25.1</v>
       </c>
     </row>
@@ -6296,25 +6294,25 @@
       <c r="A12" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="53">
+      <c r="B12" s="34">
         <v>40</v>
       </c>
-      <c r="C12" s="53">
+      <c r="C12" s="34">
         <v>41.8</v>
       </c>
-      <c r="D12" s="53">
+      <c r="D12" s="34">
         <v>35.799999999999997</v>
       </c>
-      <c r="E12" s="53">
+      <c r="E12" s="34">
         <v>43.4</v>
       </c>
-      <c r="F12" s="53">
+      <c r="F12" s="34">
         <v>44.5</v>
       </c>
-      <c r="G12" s="53">
+      <c r="G12" s="34">
         <v>38.299999999999997</v>
       </c>
-      <c r="H12" s="53">
+      <c r="H12" s="34">
         <v>38.9</v>
       </c>
     </row>
@@ -6322,25 +6320,25 @@
       <c r="A13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="53">
+      <c r="B13" s="34">
         <v>34.6</v>
       </c>
-      <c r="C13" s="53">
+      <c r="C13" s="34">
         <v>34.5</v>
       </c>
-      <c r="D13" s="53">
+      <c r="D13" s="34">
         <v>36.6</v>
       </c>
-      <c r="E13" s="53">
+      <c r="E13" s="34">
         <v>37.4</v>
       </c>
-      <c r="F13" s="53">
+      <c r="F13" s="34">
         <v>31.9</v>
       </c>
-      <c r="G13" s="53">
+      <c r="G13" s="34">
         <v>27.5</v>
       </c>
-      <c r="H13" s="53">
+      <c r="H13" s="34">
         <v>30.9</v>
       </c>
     </row>
@@ -6348,25 +6346,25 @@
       <c r="A14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="53">
+      <c r="B14" s="34">
         <v>32.799999999999997</v>
       </c>
-      <c r="C14" s="53">
+      <c r="C14" s="34">
         <v>35.4</v>
       </c>
-      <c r="D14" s="53">
+      <c r="D14" s="34">
         <v>31.4</v>
       </c>
-      <c r="E14" s="53">
+      <c r="E14" s="34">
         <v>27</v>
       </c>
-      <c r="F14" s="53">
+      <c r="F14" s="34">
         <v>29.1</v>
       </c>
-      <c r="G14" s="53">
+      <c r="G14" s="34">
         <v>32.799999999999997</v>
       </c>
-      <c r="H14" s="53">
+      <c r="H14" s="34">
         <v>29.7</v>
       </c>
     </row>
@@ -6378,7 +6376,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="11.42578125" style="10" customWidth="1"/>
@@ -6406,7 +6404,7 @@
         <v>29</v>
       </c>
       <c r="C2" s="11">
-        <v>475539.40286010271</v>
+        <v>475537.70083741978</v>
       </c>
       <c r="D2" s="11">
         <v>460369.44223294902</v>
@@ -6420,7 +6418,7 @@
         <v>30</v>
       </c>
       <c r="C3" s="11">
-        <v>470354.11948447995</v>
+        <v>470384.93700198462</v>
       </c>
       <c r="D3" s="11">
         <v>514395.68177236198</v>
@@ -6434,7 +6432,7 @@
         <v>31</v>
       </c>
       <c r="C4" s="11">
-        <v>493797.37820779701</v>
+        <v>493754.15344490833</v>
       </c>
       <c r="D4" s="11">
         <v>481151.97994350799</v>
@@ -6448,7 +6446,7 @@
         <v>32</v>
       </c>
       <c r="C5" s="11">
-        <v>500769.87964556657</v>
+        <v>500783.98891432083</v>
       </c>
       <c r="D5" s="11">
         <v>484543.67687656201</v>
@@ -6462,7 +6460,7 @@
         <v>29</v>
       </c>
       <c r="C6" s="11">
-        <v>515285.82226785243</v>
+        <v>515273.14326492086</v>
       </c>
       <c r="D6" s="11">
         <v>493602.53057785501</v>
@@ -6476,7 +6474,7 @@
         <v>30</v>
       </c>
       <c r="C7" s="11">
-        <v>526591.9714851937</v>
+        <v>526633.56741282518</v>
       </c>
       <c r="D7" s="11">
         <v>581668.24987960199</v>
@@ -6490,7 +6488,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="11">
-        <v>530024.96916142374</v>
+        <v>529981.23609597038</v>
       </c>
       <c r="D8" s="11">
         <v>514697.78950542799</v>
@@ -6504,7 +6502,7 @@
         <v>32</v>
       </c>
       <c r="C9" s="11">
-        <v>540321.007099187</v>
+        <v>540335.82323994022</v>
       </c>
       <c r="D9" s="11">
         <v>522255.20005077199</v>
@@ -6518,7 +6516,7 @@
         <v>29</v>
       </c>
       <c r="C10" s="11">
-        <v>554468.16211025103</v>
+        <v>554470.06232565292</v>
       </c>
       <c r="D10" s="11">
         <v>532348.21201691695</v>
@@ -6532,7 +6530,7 @@
         <v>30</v>
       </c>
       <c r="C11" s="11">
-        <v>561434.67786953063</v>
+        <v>561452.24888728443</v>
       </c>
       <c r="D11" s="11">
         <v>614076.39260854397</v>
@@ -6546,7 +6544,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="11">
-        <v>576815.72098068486</v>
+        <v>576782.70385081007</v>
       </c>
       <c r="D12" s="11">
         <v>562978.96562687703</v>
@@ -6560,7 +6558,7 @@
         <v>32</v>
       </c>
       <c r="C13" s="11">
-        <v>589479.05592245981</v>
+        <v>589492.60181917867</v>
       </c>
       <c r="D13" s="11">
         <v>572794.04663058801</v>
@@ -6574,7 +6572,7 @@
         <v>29</v>
       </c>
       <c r="C14" s="11">
-        <v>603416.48185863218</v>
+        <v>603422.35992299067</v>
       </c>
       <c r="D14" s="11">
         <v>576846.88569942699</v>
@@ -6588,7 +6586,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="11">
-        <v>616299.39312501706</v>
+        <v>616317.4495607412</v>
       </c>
       <c r="D15" s="11">
         <v>674620.563006485</v>
@@ -6602,7 +6600,7 @@
         <v>31</v>
       </c>
       <c r="C16" s="11">
-        <v>624352.58868411044</v>
+        <v>624326.03693504655</v>
       </c>
       <c r="D16" s="11">
         <v>610425.69401485403</v>
@@ -6616,7 +6614,7 @@
         <v>32</v>
       </c>
       <c r="C17" s="11">
-        <v>643701.5469166023</v>
+        <v>643704.16416558449</v>
       </c>
       <c r="D17" s="11">
         <v>625876.867863597</v>
@@ -6630,7 +6628,7 @@
         <v>29</v>
       </c>
       <c r="C18" s="11">
-        <v>650062.83279971546</v>
+        <v>650049.66076436755</v>
       </c>
       <c r="D18" s="11">
         <v>616720.35706447798</v>
@@ -6644,7 +6642,7 @@
         <v>30</v>
       </c>
       <c r="C19" s="11">
-        <v>653269.76138485561</v>
+        <v>653316.47297766595</v>
       </c>
       <c r="D19" s="11">
         <v>711405.50045523304</v>
@@ -6658,7 +6656,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="11">
-        <v>657936.93255261565</v>
+        <v>657901.41737708577</v>
       </c>
       <c r="D20" s="11">
         <v>647087.95974249404</v>
@@ -6672,7 +6670,7 @@
         <v>32</v>
       </c>
       <c r="C21" s="11">
-        <v>627435.11222766025</v>
+        <v>627437.08784572734</v>
       </c>
       <c r="D21" s="11">
         <v>613490.82170264097</v>
@@ -6686,7 +6684,7 @@
         <v>29</v>
       </c>
       <c r="C22" s="11">
-        <v>604739.79905993817</v>
+        <v>604752.35374212195</v>
       </c>
       <c r="D22" s="11">
         <v>578553.04424240498</v>
@@ -6700,7 +6698,7 @@
         <v>30</v>
       </c>
       <c r="C23" s="11">
-        <v>590902.23142847931</v>
+        <v>590914.16723537177</v>
       </c>
       <c r="D23" s="11">
         <v>631197.75186006899</v>
@@ -6714,7 +6712,7 @@
         <v>31</v>
       </c>
       <c r="C24" s="11">
-        <v>614035.54343456146</v>
+        <v>614002.6808783242</v>
       </c>
       <c r="D24" s="11">
         <v>610519.85461172694</v>
@@ -6728,7 +6726,7 @@
         <v>32</v>
       </c>
       <c r="C25" s="11">
-        <v>625813.93172851868</v>
+        <v>625822.30379567994</v>
       </c>
       <c r="D25" s="11">
         <v>615220.85493729694</v>
@@ -6742,7 +6740,7 @@
         <v>29</v>
       </c>
       <c r="C26" s="11">
-        <v>644901.88693182275</v>
+        <v>644914.26862490014</v>
       </c>
       <c r="D26" s="11">
         <v>611607.33658973</v>
@@ -6756,7 +6754,7 @@
         <v>30</v>
       </c>
       <c r="C27" s="11">
-        <v>673704.24691340048</v>
+        <v>673737.21582743723</v>
       </c>
       <c r="D27" s="11">
         <v>733730.773968903</v>
@@ -6770,7 +6768,7 @@
         <v>31</v>
       </c>
       <c r="C28" s="11">
-        <v>677196.1138942315</v>
+        <v>677161.17717197642</v>
       </c>
       <c r="D28" s="11">
         <v>668566.50948898599</v>
@@ -6784,7 +6782,7 @@
         <v>32</v>
       </c>
       <c r="C29" s="11">
-        <v>686292.47002773837</v>
+        <v>686282.05614288046</v>
       </c>
       <c r="D29" s="11">
         <v>668190.097719574</v>
@@ -6798,7 +6796,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="11">
-        <v>702715.18731246202</v>
+        <v>702704.57459265646</v>
       </c>
       <c r="D30" s="11">
         <v>662325.58597269503</v>
@@ -6812,7 +6810,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="11">
-        <v>709752.09900164558</v>
+        <v>709774.23296673689</v>
       </c>
       <c r="D31" s="11">
         <v>766332.95457161299</v>
@@ -6826,7 +6824,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="11">
-        <v>715352.50699214835</v>
+        <v>715335.84050676052</v>
       </c>
       <c r="D32" s="11">
         <v>711417.39193010505</v>
@@ -6840,7 +6838,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="11">
-        <v>715306.59557615174</v>
+        <v>715311.74081625242</v>
       </c>
       <c r="D33" s="11">
         <v>703050.45640799298</v>
@@ -6854,7 +6852,7 @@
         <v>29</v>
       </c>
       <c r="C34" s="11">
-        <v>707988.22133292514</v>
+        <v>707996.19507410086</v>
       </c>
       <c r="D34" s="11">
         <v>672685.993630504</v>
@@ -6868,7 +6866,7 @@
         <v>30</v>
       </c>
       <c r="C35" s="11">
-        <v>683985.42306130065</v>
+        <v>683979.96524977789</v>
       </c>
       <c r="D35" s="11">
         <v>730838.27259277599</v>
@@ -6882,7 +6880,7 @@
         <v>31</v>
       </c>
       <c r="C36" s="11">
-        <v>705109.9934384583</v>
+        <v>705104.40650262148</v>
       </c>
       <c r="D36" s="11">
         <v>703461.65253019601</v>
@@ -6896,7 +6894,7 @@
         <v>32</v>
       </c>
       <c r="C37" s="11">
-        <v>716860.32000311208</v>
+        <v>716863.39100929687</v>
       </c>
       <c r="D37" s="11">
         <v>706958.03908231901</v>
@@ -6910,7 +6908,7 @@
         <v>29</v>
       </c>
       <c r="C38" s="11">
-        <v>716958.91356570437</v>
+        <v>716924.96376811771</v>
       </c>
       <c r="D38" s="11">
         <v>677085.52917315101</v>
@@ -6924,7 +6922,7 @@
         <v>30</v>
       </c>
       <c r="C39" s="11">
-        <v>721290.34819069924</v>
+        <v>721306.98379114177</v>
       </c>
       <c r="D39" s="11">
         <v>776486.60279942001</v>
@@ -6938,7 +6936,7 @@
         <v>31</v>
       </c>
       <c r="C40" s="11">
-        <v>725228.86057766667</v>
+        <v>725233.0951662421</v>
       </c>
       <c r="D40" s="11">
         <v>721458.94421618199</v>
@@ -6952,7 +6950,7 @@
         <v>32</v>
       </c>
       <c r="C41" s="11">
-        <v>718150.29887718929</v>
+        <v>718163.37848575902</v>
       </c>
       <c r="D41" s="11">
         <v>706597.34502250701</v>
@@ -6966,7 +6964,7 @@
         <v>29</v>
       </c>
       <c r="C42" s="11">
-        <v>707604.64972170733</v>
+        <v>707619.72920730279</v>
       </c>
       <c r="D42" s="11">
         <v>671066.04663506302</v>
@@ -6980,7 +6978,7 @@
         <v>30</v>
       </c>
       <c r="C43" s="11">
-        <v>703288.51850467571</v>
+        <v>703285.49932575063</v>
       </c>
       <c r="D43" s="11">
         <v>760576.86834800395</v>
@@ -6994,7 +6992,7 @@
         <v>31</v>
       </c>
       <c r="C44" s="11">
-        <v>697226.21978834714</v>
+        <v>697218.971951521</v>
       </c>
       <c r="D44" s="11">
         <v>690879.79825168301</v>
@@ -7008,7 +7006,7 @@
         <v>32</v>
       </c>
       <c r="C45" s="11">
-        <v>701104.79583873064</v>
+        <v>701099.98336888768</v>
       </c>
       <c r="D45" s="11">
         <v>686701.47061871097</v>
@@ -7022,7 +7020,7 @@
         <v>29</v>
       </c>
       <c r="C46" s="11">
-        <v>711401.44068145636</v>
+        <v>711402.46662486251</v>
       </c>
       <c r="D46" s="11">
         <v>672749.81139169901</v>
@@ -7036,7 +7034,7 @@
         <v>30</v>
       </c>
       <c r="C47" s="11">
-        <v>727767.46053102415</v>
+        <v>727785.32360902661</v>
       </c>
       <c r="D47" s="11">
         <v>791235.96554166998</v>
@@ -7050,7 +7048,7 @@
         <v>31</v>
       </c>
       <c r="C48" s="11">
-        <v>727494.47701461555</v>
+        <v>727484.43682691152</v>
       </c>
       <c r="D48" s="11">
         <v>718281.26544978202</v>
@@ -7064,7 +7062,7 @@
         <v>32</v>
       </c>
       <c r="C49" s="11">
-        <v>719285.20832506299</v>
+        <v>719276.35949135688</v>
       </c>
       <c r="D49" s="11">
         <v>703681.54416900803</v>
@@ -7078,7 +7076,7 @@
         <v>29</v>
       </c>
       <c r="C50" s="11">
-        <v>712710.63575714745</v>
+        <v>712727.30457145628</v>
       </c>
       <c r="D50" s="11">
         <v>677652.08911570301</v>
@@ -7092,7 +7090,7 @@
         <v>30</v>
       </c>
       <c r="C51" s="11">
-        <v>701267.87546475301</v>
+        <v>701302.65391580248</v>
       </c>
       <c r="D51" s="11">
         <v>760703.28015165601</v>
@@ -7106,7 +7104,7 @@
         <v>31</v>
       </c>
       <c r="C52" s="11">
-        <v>703825.31306672294</v>
+        <v>703800.64895787265</v>
       </c>
       <c r="D52" s="11">
         <v>694382.47577623103</v>
@@ -7120,7 +7118,7 @@
         <v>32</v>
       </c>
       <c r="C53" s="11">
-        <v>708107.57010202378</v>
+        <v>708080.78694551589</v>
       </c>
       <c r="D53" s="11">
         <v>693173.54934705805</v>
@@ -7134,7 +7132,7 @@
         <v>29</v>
       </c>
       <c r="C54" s="11">
-        <v>714000.68213478185</v>
+        <v>714073.96772732539</v>
       </c>
       <c r="D54" s="11">
         <v>681444.76611022197</v>
@@ -7148,7 +7146,7 @@
         <v>30</v>
       </c>
       <c r="C55" s="11">
-        <v>722206.78209549456</v>
+        <v>722256.71770503907</v>
       </c>
       <c r="D55" s="11">
         <v>778401.67644931702</v>
@@ -7162,7 +7160,7 @@
         <v>31</v>
       </c>
       <c r="C56" s="11">
-        <v>731022.65780373593</v>
+        <v>730990.52731986262</v>
       </c>
       <c r="D56" s="11">
         <v>721120.42685279401</v>
@@ -7176,7 +7174,7 @@
         <v>32</v>
       </c>
       <c r="C57" s="11">
-        <v>738329.66901728406</v>
+        <v>738238.57829906943</v>
       </c>
       <c r="D57" s="11">
         <v>724592.92163896305</v>
@@ -7190,7 +7188,7 @@
         <v>29</v>
       </c>
       <c r="C58" s="11">
-        <v>735269.26388700691</v>
+        <v>735391.8994718258</v>
       </c>
       <c r="D58" s="11">
         <v>707324.26805721398</v>
@@ -7204,7 +7202,7 @@
         <v>30</v>
       </c>
       <c r="C59" s="11">
-        <v>702794.19038738846</v>
+        <v>702876.70139706763</v>
       </c>
       <c r="D59" s="11">
         <v>747428.29995457502</v>
@@ -7218,7 +7216,7 @@
         <v>31</v>
       </c>
       <c r="C60" s="11">
-        <v>700585.06179718161</v>
+        <v>700556.41071643296</v>
       </c>
       <c r="D60" s="11">
         <v>696101.58352180803</v>
@@ -7232,7 +7230,7 @@
         <v>32</v>
       </c>
       <c r="C61" s="11">
-        <v>690861.25584647327</v>
+        <v>690684.76033272361</v>
       </c>
       <c r="D61" s="11">
         <v>678655.62038445403</v>
@@ -7246,7 +7244,7 @@
         <v>29</v>
       </c>
       <c r="C62" s="11">
-        <v>690992.53890621837</v>
+        <v>691181.1710735294</v>
       </c>
       <c r="D62">
         <v>665848.71529970889</v>
@@ -7260,7 +7258,7 @@
         <v>30</v>
       </c>
       <c r="C63" s="11">
-        <v>697721.48697133223</v>
+        <v>697844.86357814202</v>
       </c>
       <c r="D63">
         <v>751784.46077713254</v>
@@ -7274,7 +7272,7 @@
         <v>31</v>
       </c>
       <c r="C64" s="11">
-        <v>697245.70141462015</v>
+        <v>697203.38606212521</v>
       </c>
       <c r="D64">
         <v>683900.89855257841</v>
@@ -7288,7 +7286,7 @@
         <v>32</v>
       </c>
       <c r="C65" s="11">
-        <v>686935.48705966782</v>
+        <v>686665.79363804066</v>
       </c>
       <c r="D65">
         <v>671361.13972242002</v>
@@ -7302,7 +7300,7 @@
         <v>29</v>
       </c>
       <c r="C66" s="10">
-        <v>657234.36724165711</v>
+        <v>657389.34307522234</v>
       </c>
       <c r="D66" s="10">
         <v>632389.35353461001</v>
@@ -7316,7 +7314,7 @@
         <v>30</v>
       </c>
       <c r="C67" s="10">
-        <v>562000.89823407296</v>
+        <v>562179.99566802813</v>
       </c>
       <c r="D67" s="10">
         <v>609379.98946480127</v>
@@ -7330,7 +7328,7 @@
         <v>31</v>
       </c>
       <c r="C68" s="10">
-        <v>623856.36323480471</v>
+        <v>623774.81706188689</v>
       </c>
       <c r="D68" s="10">
         <v>614192.47840422287</v>
@@ -7344,7 +7342,7 @@
         <v>32</v>
       </c>
       <c r="C69" s="10">
-        <v>655273.51589104964</v>
+        <v>655020.98879644717</v>
       </c>
       <c r="D69" s="10">
         <v>642403.32319795026</v>
@@ -7358,7 +7356,7 @@
         <v>29</v>
       </c>
       <c r="C70" s="10">
-        <v>677518.09192361217</v>
+        <v>677641.85107030324</v>
       </c>
       <c r="D70">
         <v>652831.97670632158</v>
@@ -7372,7 +7370,7 @@
         <v>30</v>
       </c>
       <c r="C71" s="10">
-        <v>678667.84323796758</v>
+        <v>678936.36360114603</v>
       </c>
       <c r="D71">
         <v>723516.62249067484</v>
@@ -7386,7 +7384,7 @@
         <v>31</v>
       </c>
       <c r="C72" s="10">
-        <v>693508.41694142157</v>
+        <v>693434.13508999697</v>
       </c>
       <c r="D72" s="10">
         <v>686756.46782667423</v>
@@ -7400,7 +7398,7 @@
         <v>32</v>
       </c>
       <c r="C73" s="10">
-        <v>709545.38403278519</v>
+        <v>709227.38637434016</v>
       </c>
       <c r="D73" s="10">
         <v>696134.66911211505</v>
@@ -7414,7 +7412,7 @@
         <v>29</v>
       </c>
       <c r="C74" s="10">
-        <v>726994.4331088519</v>
+        <v>727024.01166009402</v>
       </c>
       <c r="D74">
         <v>697625.28466635814</v>
@@ -7428,7 +7426,7 @@
         <v>30</v>
       </c>
       <c r="C75" s="10">
-        <v>741461.96753675886</v>
+        <v>741845.29873761034</v>
       </c>
       <c r="D75">
         <v>782338.62853373506</v>
@@ -7442,7 +7440,7 @@
         <v>31</v>
       </c>
       <c r="C76" s="10">
-        <v>735869.56325702253</v>
+        <v>735700.58443679963</v>
       </c>
       <c r="D76" s="10">
         <v>732662.16387550125</v>
@@ -7456,7 +7454,7 @@
         <v>32</v>
       </c>
       <c r="C77" s="10">
-        <v>721040.57100169931</v>
+        <v>720796.64006982953</v>
       </c>
       <c r="D77" s="10">
         <v>712740.45782873826</v>
@@ -7470,7 +7468,7 @@
         <v>29</v>
       </c>
       <c r="C78" s="10">
-        <v>729079.81570524594</v>
+        <v>728927.34399396658</v>
       </c>
       <c r="D78" s="10">
         <v>704009.03517700161</v>
@@ -7485,7 +7483,7 @@
         <v>30</v>
       </c>
       <c r="C79" s="10">
-        <v>709842.35270039842</v>
+        <v>710090.35214944521</v>
       </c>
       <c r="D79" s="10">
         <v>738128.41122730402</v>
@@ -7500,7 +7498,7 @@
         <v>31</v>
       </c>
       <c r="C80" s="10">
-        <v>725214.64378983236</v>
+        <v>725224.98127715138</v>
       </c>
       <c r="D80" s="10">
         <v>728542.25584748655</v>
@@ -7515,7 +7513,7 @@
         <v>32</v>
       </c>
       <c r="C81" s="10">
-        <v>707086.08875387569</v>
+        <v>706980.22352878936</v>
       </c>
       <c r="D81" s="10">
         <v>700543.19869756</v>
@@ -7529,7 +7527,7 @@
         <v>29</v>
       </c>
       <c r="C82" s="10">
-        <v>694486.09954866616</v>
+        <v>694139.06625708297</v>
       </c>
       <c r="D82" s="10">
         <v>668219.6308270538</v>
@@ -7543,7 +7541,7 @@
         <v>30</v>
       </c>
       <c r="C83" s="10">
-        <v>691468.75067544018</v>
+        <v>691368.83663512988</v>
       </c>
       <c r="D83">
         <v>729909.36871982319</v>
@@ -7557,7 +7555,7 @@
         <v>31</v>
       </c>
       <c r="C84" s="10">
-        <v>716166.17456055968</v>
+        <v>716468.58381510247</v>
       </c>
       <c r="D84">
         <v>714299.21795624029</v>
@@ -7571,7 +7569,7 @@
         <v>32</v>
       </c>
       <c r="C85" s="10">
-        <v>729830.51344938693</v>
+        <v>729975.05152673856</v>
       </c>
       <c r="D85" s="10">
         <v>719523.32073093485</v>
@@ -7585,7 +7583,7 @@
         <v>29</v>
       </c>
       <c r="C86" s="10">
-        <v>735468.22118616325</v>
+        <v>734825.66564565257</v>
       </c>
       <c r="D86" s="10">
         <v>709095.12469662423</v>
@@ -7599,7 +7597,7 @@
         <v>30</v>
       </c>
       <c r="C87" s="10">
-        <v>737703.22646665608</v>
+        <v>737286.39291679149</v>
       </c>
       <c r="D87" s="10">
         <v>777482.55560690013</v>
@@ -7613,7 +7611,7 @@
         <v>31</v>
       </c>
       <c r="C88" s="10">
-        <v>738582.97927448282</v>
+        <v>739394.27731973841</v>
       </c>
       <c r="D88">
         <v>737135.06767770939</v>
@@ -7627,7 +7625,7 @@
         <v>32</v>
       </c>
       <c r="C89" s="10">
-        <v>747160.42718325544</v>
+        <v>747408.51828521001</v>
       </c>
       <c r="D89">
         <v>735202.10550800152</v>
@@ -7641,10 +7639,24 @@
         <v>29</v>
       </c>
       <c r="C90" s="10">
-        <v>752727.87372926541</v>
-      </c>
-      <c r="D90" s="10">
-        <v>725600.2445682534</v>
+        <v>752422.5367911529</v>
+      </c>
+      <c r="D90">
+        <v>726163.281251173</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="10">
+        <v>2026</v>
+      </c>
+      <c r="B91" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C91" s="10">
+        <v>747969.90325672424</v>
+      </c>
+      <c r="D91">
+        <v>792800.34147831588</v>
       </c>
     </row>
   </sheetData>
@@ -8450,14 +8462,14 @@
         <v>70</v>
       </c>
       <c r="B2" s="46">
-        <v>10131.835788459999</v>
+        <v>11730.33175329</v>
       </c>
       <c r="C2" s="46">
-        <v>12382.20280524</v>
+        <v>14332.557392840001</v>
       </c>
       <c r="D2" s="27">
         <f>B2-C2</f>
-        <v>-2250.367016780001</v>
+        <v>-2602.2256395500008</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -8465,14 +8477,14 @@
         <v>203</v>
       </c>
       <c r="B3" s="42">
-        <v>7386.56491147</v>
+        <v>8577.9098430699996</v>
       </c>
       <c r="C3" s="42">
-        <v>9135.5407090499994</v>
+        <v>10629.94907769</v>
       </c>
       <c r="D3" s="27">
         <f t="shared" ref="D3:D27" si="0">B3-C3</f>
-        <v>-1748.9757975799994</v>
+        <v>-2052.0392346200006</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -8480,14 +8492,14 @@
         <v>208</v>
       </c>
       <c r="B4" s="42">
-        <v>1046.4819220100001</v>
+        <v>1199.62775519</v>
       </c>
       <c r="C4" s="42">
-        <v>2905.88218284</v>
+        <v>3296.06363272</v>
       </c>
       <c r="D4" s="27">
         <f t="shared" si="0"/>
-        <v>-1859.40026083</v>
+        <v>-2096.4358775299997</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -8495,14 +8507,14 @@
         <v>209</v>
       </c>
       <c r="B5" s="42">
-        <v>1352.6515661799999</v>
+        <v>1505.5014949900001</v>
       </c>
       <c r="C5" s="42">
-        <v>335.50739291000002</v>
+        <v>400.64444258999998</v>
       </c>
       <c r="D5" s="27">
         <f t="shared" si="0"/>
-        <v>1017.1441732699999</v>
+        <v>1104.8570524000002</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -8510,14 +8522,14 @@
         <v>72</v>
       </c>
       <c r="B6" s="46">
-        <v>7276.7667382099999</v>
+        <v>8316.7128498999991</v>
       </c>
       <c r="C6" s="46">
-        <v>1336.49858073</v>
+        <v>1561.26989688</v>
       </c>
       <c r="D6" s="27">
         <f t="shared" si="0"/>
-        <v>5940.2681574799999</v>
+        <v>6755.4429530199995</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -8525,14 +8537,14 @@
         <v>71</v>
       </c>
       <c r="B7" s="42">
-        <v>3787.38927302</v>
+        <v>4288.9319074699997</v>
       </c>
       <c r="C7" s="42">
-        <v>522.54152991000001</v>
+        <v>575.48966665</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" si="0"/>
-        <v>3264.84774311</v>
+        <v>3713.4422408199998</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -8540,14 +8552,14 @@
         <v>204</v>
       </c>
       <c r="B8" s="42">
-        <v>1741.6900650600001</v>
+        <v>2002.80556398</v>
       </c>
       <c r="C8" s="42">
-        <v>175.76956447000001</v>
+        <v>200.23070425</v>
       </c>
       <c r="D8" s="27">
         <f t="shared" si="0"/>
-        <v>1565.9205005900001</v>
+        <v>1802.5748597300001</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -8555,14 +8567,14 @@
         <v>175</v>
       </c>
       <c r="B9" s="46">
-        <v>7243.4021109400001</v>
+        <v>8171.8416171899999</v>
       </c>
       <c r="C9" s="46">
-        <v>5225.90957196</v>
+        <v>5900.1284501500004</v>
       </c>
       <c r="D9" s="27">
         <f t="shared" si="0"/>
-        <v>2017.4925389800001</v>
+        <v>2271.7131670399995</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -8570,14 +8582,14 @@
         <v>205</v>
       </c>
       <c r="B10" s="42">
-        <v>5970.7614276200002</v>
+        <v>6691.4666677699997</v>
       </c>
       <c r="C10" s="42">
-        <v>3967.0999705899999</v>
+        <v>4529.8080052300002</v>
       </c>
       <c r="D10" s="27">
         <f t="shared" si="0"/>
-        <v>2003.6614570300003</v>
+        <v>2161.6586625399996</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -8585,14 +8597,14 @@
         <v>176</v>
       </c>
       <c r="B11" s="46">
-        <v>5199.1678182699998</v>
+        <v>6222.0785865199996</v>
       </c>
       <c r="C11" s="46">
-        <v>5782.4787789499997</v>
+        <v>6625.6950472400003</v>
       </c>
       <c r="D11" s="27">
         <f t="shared" si="0"/>
-        <v>-583.31096067999988</v>
+        <v>-403.61646072000076</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -8600,14 +8612,14 @@
         <v>212</v>
       </c>
       <c r="B12" s="42">
-        <v>659.46119262000002</v>
+        <v>769.16592227000001</v>
       </c>
       <c r="C12" s="42">
-        <v>1798.04473865</v>
+        <v>2053.1686061700002</v>
       </c>
       <c r="D12" s="27">
         <f t="shared" si="0"/>
-        <v>-1138.58354603</v>
+        <v>-1284.0026839000002</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -8615,14 +8627,14 @@
         <v>213</v>
       </c>
       <c r="B13" s="42">
-        <v>923.75633140000002</v>
+        <v>1128.9283964700001</v>
       </c>
       <c r="C13" s="42">
-        <v>593.88788952000004</v>
+        <v>687.46461611999996</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>329.86844187999998</v>
+        <v>441.46378035000009</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -8630,14 +8642,14 @@
         <v>214</v>
       </c>
       <c r="B14" s="42">
-        <v>597.18803424999999</v>
+        <v>770.90505522000001</v>
       </c>
       <c r="C14" s="42">
-        <v>878.77091515999996</v>
+        <v>1025.9636580599999</v>
       </c>
       <c r="D14" s="27">
         <f t="shared" si="0"/>
-        <v>-281.58288090999997</v>
+        <v>-255.05860283999993</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -8645,14 +8657,14 @@
         <v>215</v>
       </c>
       <c r="B15" s="42">
-        <v>1135.45100806</v>
+        <v>1356.0770490699999</v>
       </c>
       <c r="C15" s="42">
-        <v>190.25197933000001</v>
+        <v>215.60331056999999</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>945.19902873000001</v>
+        <v>1140.4737384999999</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -8660,14 +8672,14 @@
         <v>74</v>
       </c>
       <c r="B16" s="46">
-        <v>5589.1728557099996</v>
+        <v>6155.1991863900002</v>
       </c>
       <c r="C16" s="46">
-        <v>9494.7219496399994</v>
+        <v>11229.9276689</v>
       </c>
       <c r="D16" s="27">
         <f t="shared" si="0"/>
-        <v>-3905.5490939299998</v>
+        <v>-5074.7284825099996</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -8675,14 +8687,14 @@
         <v>75</v>
       </c>
       <c r="B17" s="46">
-        <v>3684.9481077599999</v>
+        <v>4276.45312431</v>
       </c>
       <c r="C17" s="46">
-        <v>649.82246679000002</v>
+        <v>779.18460789999995</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>3035.1256409699999</v>
+        <v>3497.2685164100003</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -8690,14 +8702,14 @@
         <v>73</v>
       </c>
       <c r="B18" s="46">
-        <v>5318.7616484999999</v>
+        <v>6316.4825914599996</v>
       </c>
       <c r="C18" s="46">
-        <v>2310.8556745300002</v>
+        <v>2661.3959148200001</v>
       </c>
       <c r="D18" s="27">
         <f t="shared" si="0"/>
-        <v>3007.9059739699996</v>
+        <v>3655.0866766399995</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -8705,14 +8717,14 @@
         <v>207</v>
       </c>
       <c r="B19" s="42">
-        <v>863.06267104999995</v>
+        <v>1035.20953153</v>
       </c>
       <c r="C19" s="42">
-        <v>238.04602537</v>
+        <v>287.44898253000002</v>
       </c>
       <c r="D19" s="27">
         <f t="shared" si="0"/>
-        <v>625.01664568000001</v>
+        <v>747.76054900000008</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -8720,14 +8732,14 @@
         <v>210</v>
       </c>
       <c r="B20" s="42">
-        <v>909.10152768</v>
+        <v>1170.8101533199999</v>
       </c>
       <c r="C20" s="42">
-        <v>134.54632391000001</v>
+        <v>151.96947852</v>
       </c>
       <c r="D20" s="27">
         <f t="shared" si="0"/>
-        <v>774.55520376999993</v>
+        <v>1018.8406748</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -8735,14 +8747,14 @@
         <v>211</v>
       </c>
       <c r="B21" s="42">
-        <v>991.09674127999995</v>
+        <v>1136.0953787399999</v>
       </c>
       <c r="C21" s="42">
-        <v>1185.1922510899999</v>
+        <v>1349.22044682</v>
       </c>
       <c r="D21" s="27">
         <f t="shared" si="0"/>
-        <v>-194.09550980999995</v>
+        <v>-213.12506808000012</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -8750,14 +8762,14 @@
         <v>206</v>
       </c>
       <c r="B22" s="42">
-        <v>2104.22535883</v>
+        <v>2421.13608991</v>
       </c>
       <c r="C22" s="42">
-        <v>570.53177382000001</v>
+        <v>669.25282884000001</v>
       </c>
       <c r="D22" s="27">
         <f t="shared" si="0"/>
-        <v>1533.6935850099999</v>
+        <v>1751.8832610700001</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -8765,14 +8777,14 @@
         <v>76</v>
       </c>
       <c r="B23" s="46">
-        <v>2974.4506729999998</v>
+        <v>3400.7110296199999</v>
       </c>
       <c r="C23" s="46">
-        <v>268.65412280999999</v>
+        <v>325.37604098000003</v>
       </c>
       <c r="D23" s="27">
         <f t="shared" si="0"/>
-        <v>2705.7965501899998</v>
+        <v>3075.3349886399997</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -8780,14 +8792,14 @@
         <v>77</v>
       </c>
       <c r="B24" s="46">
-        <v>2576.3643842800002</v>
+        <v>2723.3428194799999</v>
       </c>
       <c r="C24" s="46">
-        <v>367.98612315999998</v>
+        <v>427.87939122</v>
       </c>
       <c r="D24" s="27">
         <f t="shared" si="0"/>
-        <v>2208.3782611200004</v>
+        <v>2295.46342826</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -8795,14 +8807,14 @@
         <v>78</v>
       </c>
       <c r="B25" s="46">
-        <v>199.64993278</v>
+        <v>229.78354913999999</v>
       </c>
       <c r="C25" s="46">
-        <v>126.95507979999999</v>
+        <v>136.89460957</v>
       </c>
       <c r="D25" s="27">
         <f t="shared" si="0"/>
-        <v>72.694852980000007</v>
+        <v>92.888939569999991</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -8810,14 +8822,14 @@
         <v>79</v>
       </c>
       <c r="B26" s="46">
-        <v>606.94943167999998</v>
+        <v>755.64002840000001</v>
       </c>
       <c r="C26" s="46">
-        <v>201.79184792000001</v>
+        <v>226.26251718</v>
       </c>
       <c r="D26" s="27">
         <f t="shared" si="0"/>
-        <v>405.15758375999997</v>
+        <v>529.37751121999997</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -8825,14 +8837,14 @@
         <v>80</v>
       </c>
       <c r="B27" s="47">
-        <v>7563.7167973200003</v>
+        <v>8949.1916499800009</v>
       </c>
       <c r="C27" s="47">
-        <v>4137.7659778699999</v>
+        <v>4792.11866758</v>
       </c>
       <c r="D27" s="27">
         <f t="shared" si="0"/>
-        <v>3425.9508194500004</v>
+        <v>4157.0729824000009</v>
       </c>
     </row>
   </sheetData>
@@ -8862,7 +8874,7 @@
         <v>172</v>
       </c>
       <c r="B2" s="48">
-        <v>58365.18628691</v>
+        <v>67247.768785680004</v>
       </c>
       <c r="D2" s="29"/>
     </row>
@@ -8871,7 +8883,7 @@
         <v>168</v>
       </c>
       <c r="B3" s="48">
-        <v>14749.46763087</v>
+        <v>16480.22902545</v>
       </c>
       <c r="D3" s="29"/>
     </row>
@@ -8880,7 +8892,7 @@
         <v>121</v>
       </c>
       <c r="B4" s="49">
-        <v>18.157807630000001</v>
+        <v>20.101308509999999</v>
       </c>
       <c r="D4" s="30"/>
     </row>
@@ -8889,7 +8901,7 @@
         <v>122</v>
       </c>
       <c r="B5" s="49">
-        <v>1256.8318682199999</v>
+        <v>1468.3693771000001</v>
       </c>
       <c r="D5" s="30"/>
     </row>
@@ -8898,7 +8910,7 @@
         <v>123</v>
       </c>
       <c r="B6" s="49">
-        <v>201.09731998000001</v>
+        <v>223.15063314</v>
       </c>
       <c r="D6" s="30"/>
     </row>
@@ -8907,7 +8919,7 @@
         <v>124</v>
       </c>
       <c r="B7" s="49">
-        <v>470.26634000000001</v>
+        <v>535.44731380999997</v>
       </c>
       <c r="D7" s="30"/>
     </row>
@@ -8916,7 +8928,7 @@
         <v>125</v>
       </c>
       <c r="B8" s="49">
-        <v>509.21601561</v>
+        <v>561.20805385000006</v>
       </c>
       <c r="D8" s="30"/>
     </row>
@@ -8925,7 +8937,7 @@
         <v>126</v>
       </c>
       <c r="B9" s="49">
-        <v>8762.7264263800007</v>
+        <v>9772.09621591</v>
       </c>
       <c r="D9" s="30"/>
     </row>
@@ -8934,7 +8946,7 @@
         <v>127</v>
       </c>
       <c r="B10" s="49">
-        <v>2444.2489930800002</v>
+        <v>2662.54073986</v>
       </c>
       <c r="D10" s="30"/>
     </row>
@@ -8943,7 +8955,7 @@
         <v>128</v>
       </c>
       <c r="B11" s="49">
-        <v>156.34153777</v>
+        <v>190.99193421000001</v>
       </c>
       <c r="D11" s="30"/>
     </row>
@@ -8952,7 +8964,7 @@
         <v>129</v>
       </c>
       <c r="B12" s="49">
-        <v>60.934622490000002</v>
+        <v>70.052651049999994</v>
       </c>
       <c r="D12" s="30"/>
     </row>
@@ -8961,7 +8973,7 @@
         <v>130</v>
       </c>
       <c r="B13" s="49">
-        <v>71.689543749999999</v>
+        <v>87.533367830000003</v>
       </c>
       <c r="D13" s="30"/>
     </row>
@@ -8970,7 +8982,7 @@
         <v>131</v>
       </c>
       <c r="B14" s="49">
-        <v>670.09803132000002</v>
+        <v>748.84156416999997</v>
       </c>
       <c r="D14" s="30"/>
     </row>
@@ -8979,7 +8991,7 @@
         <v>132</v>
       </c>
       <c r="B15" s="49">
-        <v>127.85912464</v>
+        <v>139.89586600999999</v>
       </c>
       <c r="D15" s="30"/>
     </row>
@@ -8988,7 +9000,7 @@
         <v>169</v>
       </c>
       <c r="B16" s="48">
-        <v>18910.693595339999</v>
+        <v>22206.062888460001</v>
       </c>
       <c r="D16" s="29"/>
     </row>
@@ -8997,7 +9009,7 @@
         <v>133</v>
       </c>
       <c r="B17" s="49">
-        <v>3097.1531389400002</v>
+        <v>3670.0701619699998</v>
       </c>
       <c r="D17" s="30"/>
     </row>
@@ -9006,7 +9018,7 @@
         <v>134</v>
       </c>
       <c r="B18" s="49">
-        <v>181.72376378999999</v>
+        <v>208.18073641000001</v>
       </c>
       <c r="D18" s="30"/>
     </row>
@@ -9015,7 +9027,7 @@
         <v>135</v>
       </c>
       <c r="B19" s="49">
-        <v>854.0703671</v>
+        <v>977.86101798000004</v>
       </c>
       <c r="D19" s="30"/>
     </row>
@@ -9024,7 +9036,7 @@
         <v>136</v>
       </c>
       <c r="B20" s="49">
-        <v>57.90506328</v>
+        <v>67.576166659999998</v>
       </c>
       <c r="D20" s="30"/>
     </row>
@@ -9033,7 +9045,7 @@
         <v>137</v>
       </c>
       <c r="B21" s="49">
-        <v>69.489123500000005</v>
+        <v>81.563704099999995</v>
       </c>
       <c r="D21" s="30"/>
     </row>
@@ -9042,7 +9054,7 @@
         <v>138</v>
       </c>
       <c r="B22" s="49">
-        <v>109.83325639</v>
+        <v>127.5469717</v>
       </c>
       <c r="D22" s="30"/>
     </row>
@@ -9051,7 +9063,7 @@
         <v>139</v>
       </c>
       <c r="B23" s="49">
-        <v>474.87592073000002</v>
+        <v>527.70245546000001</v>
       </c>
       <c r="D23" s="30"/>
     </row>
@@ -9060,7 +9072,7 @@
         <v>140</v>
       </c>
       <c r="B24" s="49">
-        <v>6315.0275704100004</v>
+        <v>7391.6640766999999</v>
       </c>
       <c r="D24" s="30"/>
     </row>
@@ -9069,7 +9081,7 @@
         <v>141</v>
       </c>
       <c r="B25" s="49">
-        <v>222.67925025</v>
+        <v>253.92114058000001</v>
       </c>
       <c r="D25" s="30"/>
     </row>
@@ -9078,7 +9090,7 @@
         <v>142</v>
       </c>
       <c r="B26" s="49">
-        <v>620.26536309000005</v>
+        <v>722.88290491999999</v>
       </c>
       <c r="D26" s="30"/>
     </row>
@@ -9087,7 +9099,7 @@
         <v>143</v>
       </c>
       <c r="B27" s="49">
-        <v>436.22027859000002</v>
+        <v>478.13456760000003</v>
       </c>
       <c r="D27" s="30"/>
     </row>
@@ -9096,7 +9108,7 @@
         <v>144</v>
       </c>
       <c r="B28" s="49">
-        <v>5592.0888350599998</v>
+        <v>6685.94059664</v>
       </c>
       <c r="D28" s="30"/>
     </row>
@@ -9105,7 +9117,7 @@
         <v>145</v>
       </c>
       <c r="B29" s="49">
-        <v>181.02550357999999</v>
+        <v>212.31669382999999</v>
       </c>
       <c r="D29" s="30"/>
     </row>
@@ -9114,7 +9126,7 @@
         <v>146</v>
       </c>
       <c r="B30" s="49">
-        <v>205.02960447000001</v>
+        <v>238.07436966</v>
       </c>
       <c r="D30" s="30"/>
     </row>
@@ -9123,7 +9135,7 @@
         <v>147</v>
       </c>
       <c r="B31" s="49">
-        <v>78.771963679999999</v>
+        <v>91.66533622</v>
       </c>
       <c r="D31" s="30"/>
     </row>
@@ -9132,7 +9144,7 @@
         <v>148</v>
       </c>
       <c r="B32" s="49">
-        <v>414.53459248000001</v>
+        <v>470.96198802999999</v>
       </c>
       <c r="D32" s="30"/>
     </row>
@@ -9141,7 +9153,7 @@
         <v>170</v>
       </c>
       <c r="B33" s="48">
-        <v>15553.555421290001</v>
+        <v>17894.47491017</v>
       </c>
       <c r="D33" s="29"/>
     </row>
@@ -9150,7 +9162,7 @@
         <v>149</v>
       </c>
       <c r="B34" s="49">
-        <v>3533.0068182999998</v>
+        <v>4152.2687079099996</v>
       </c>
       <c r="D34" s="30"/>
     </row>
@@ -9159,7 +9171,7 @@
         <v>150</v>
       </c>
       <c r="B35" s="49">
-        <v>735.04779130999998</v>
+        <v>822.11696787999995</v>
       </c>
       <c r="D35" s="30"/>
     </row>
@@ -9168,7 +9180,7 @@
         <v>151</v>
       </c>
       <c r="B36" s="49">
-        <v>101.79144912</v>
+        <v>115.9260226</v>
       </c>
       <c r="D36" s="30"/>
     </row>
@@ -9177,7 +9189,7 @@
         <v>152</v>
       </c>
       <c r="B37" s="49">
-        <v>10.22030971</v>
+        <v>11.98579423</v>
       </c>
       <c r="D37" s="30"/>
     </row>
@@ -9186,7 +9198,7 @@
         <v>153</v>
       </c>
       <c r="B38" s="49">
-        <v>244.06434983</v>
+        <v>268.75686449</v>
       </c>
       <c r="D38" s="30"/>
     </row>
@@ -9195,7 +9207,7 @@
         <v>154</v>
       </c>
       <c r="B39" s="49">
-        <v>61.774884800000002</v>
+        <v>69.535566700000004</v>
       </c>
       <c r="D39" s="30"/>
     </row>
@@ -9204,7 +9216,7 @@
         <v>155</v>
       </c>
       <c r="B40" s="49">
-        <v>5.2625535000000001</v>
+        <v>5.6628988700000003</v>
       </c>
       <c r="D40" s="30"/>
     </row>
@@ -9213,7 +9225,7 @@
         <v>156</v>
       </c>
       <c r="B41" s="49">
-        <v>76.379257499999994</v>
+        <v>86.869893590000004</v>
       </c>
       <c r="D41" s="30"/>
     </row>
@@ -9222,7 +9234,7 @@
         <v>157</v>
       </c>
       <c r="B42" s="49">
-        <v>3237.7422759599999</v>
+        <v>3669.6649587400002</v>
       </c>
       <c r="D42" s="30"/>
     </row>
@@ -9231,7 +9243,7 @@
         <v>158</v>
       </c>
       <c r="B43" s="49">
-        <v>1660.5043017999999</v>
+        <v>1824.52611748</v>
       </c>
       <c r="D43" s="30"/>
     </row>
@@ -9240,7 +9252,7 @@
         <v>159</v>
       </c>
       <c r="B44" s="49">
-        <v>774.47669218999999</v>
+        <v>905.29051629000003</v>
       </c>
       <c r="D44" s="30"/>
     </row>
@@ -9249,7 +9261,7 @@
         <v>160</v>
       </c>
       <c r="B45" s="49">
-        <v>4621.4257138399998</v>
+        <v>5443.3517914000004</v>
       </c>
       <c r="D45" s="30"/>
     </row>
@@ -9258,7 +9270,7 @@
         <v>161</v>
       </c>
       <c r="B46" s="49">
-        <v>103.31335292</v>
+        <v>108.64312488</v>
       </c>
       <c r="D46" s="30"/>
     </row>
@@ -9267,7 +9279,7 @@
         <v>162</v>
       </c>
       <c r="B47" s="49">
-        <v>388.54567050999998</v>
+        <v>409.87568511000001</v>
       </c>
       <c r="D47" s="30"/>
     </row>
@@ -9276,7 +9288,7 @@
         <v>171</v>
       </c>
       <c r="B48" s="48">
-        <v>9151.4696394099992</v>
+        <v>10667.001961600001</v>
       </c>
       <c r="D48" s="29"/>
     </row>
@@ -9285,7 +9297,7 @@
         <v>163</v>
       </c>
       <c r="B49" s="49">
-        <v>5722.2773933500002</v>
+        <v>6625.3174199499999</v>
       </c>
       <c r="D49" s="30"/>
     </row>
@@ -9294,7 +9306,7 @@
         <v>164</v>
       </c>
       <c r="B50" s="49">
-        <v>2139.9432461699998</v>
+        <v>2563.0320099300002</v>
       </c>
       <c r="D50" s="30"/>
     </row>
@@ -9303,7 +9315,7 @@
         <v>165</v>
       </c>
       <c r="B51" s="49">
-        <v>75.096219039999994</v>
+        <v>83.760430099999994</v>
       </c>
       <c r="D51" s="30"/>
     </row>
@@ -9312,7 +9324,7 @@
         <v>166</v>
       </c>
       <c r="B52" s="42">
-        <v>932.30774222000002</v>
+        <v>1040.1389722199999</v>
       </c>
       <c r="D52" s="30"/>
     </row>
@@ -9321,7 +9333,7 @@
         <v>167</v>
       </c>
       <c r="B53" s="50">
-        <v>281.84503862999998</v>
+        <v>354.75312939999998</v>
       </c>
     </row>
   </sheetData>
@@ -9351,7 +9363,7 @@
         <v>177</v>
       </c>
       <c r="B2" s="43">
-        <v>42285.6429794</v>
+        <v>48998.690205259998</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -9359,7 +9371,7 @@
         <v>178</v>
       </c>
       <c r="B3" s="43">
-        <v>7966.5527909100001</v>
+        <v>9276.8012137000005</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -9367,7 +9379,7 @@
         <v>179</v>
       </c>
       <c r="B4" s="44">
-        <v>5703.72560419</v>
+        <v>1043.99740019</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -9375,7 +9387,7 @@
         <v>180</v>
       </c>
       <c r="B5" s="44">
-        <v>897.51211365999995</v>
+        <v>1603.6225589400001</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -9383,7 +9395,7 @@
         <v>181</v>
       </c>
       <c r="B6" s="44">
-        <v>1365.31507306</v>
+        <v>16949.051997629998</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -9391,7 +9403,7 @@
         <v>182</v>
       </c>
       <c r="B7" s="43">
-        <v>14713.917361530001</v>
+        <v>2932.0284670599999</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -9399,7 +9411,7 @@
         <v>183</v>
       </c>
       <c r="B8" s="44">
-        <v>2620.4116493299998</v>
+        <v>410.84743400999997</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -9407,7 +9419,7 @@
         <v>184</v>
       </c>
       <c r="B9" s="44">
-        <v>360.11411499000002</v>
+        <v>655.31856334999998</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -9415,7 +9427,7 @@
         <v>185</v>
       </c>
       <c r="B10" s="44">
-        <v>577.07729746999996</v>
+        <v>11583.69053021</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -9423,7 +9435,7 @@
         <v>186</v>
       </c>
       <c r="B11" s="44">
-        <v>9948.1876556099996</v>
+        <v>1367.167003</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -9431,7 +9443,7 @@
         <v>187</v>
       </c>
       <c r="B12" s="44">
-        <v>1208.1266441299999</v>
+        <v>2832.5070699500002</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -9439,7 +9451,7 @@
         <v>188</v>
       </c>
       <c r="B13" s="43">
-        <v>2298.2558634400002</v>
+        <v>297.24078580000003</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -9447,7 +9459,7 @@
         <v>189</v>
       </c>
       <c r="B14" s="44">
-        <v>229.38295342999999</v>
+        <v>2535.26628415</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -9455,7 +9467,7 @@
         <v>190</v>
       </c>
       <c r="B15" s="44">
-        <v>2068.8729100099999</v>
+        <v>8386.5318090199999</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -9463,7 +9475,7 @@
         <v>191</v>
       </c>
       <c r="B16" s="43">
-        <v>7227.0718579900004</v>
+        <v>3215.9855721600002</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -9471,7 +9483,7 @@
         <v>192</v>
       </c>
       <c r="B17" s="44">
-        <v>2773.1099563900002</v>
+        <v>445.37679042000002</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -9479,7 +9491,7 @@
         <v>193</v>
       </c>
       <c r="B18" s="44">
-        <v>375.03283696</v>
+        <v>4725.1694464399998</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -9487,7 +9499,7 @@
         <v>194</v>
       </c>
       <c r="B19" s="44">
-        <v>4078.92906464</v>
+        <v>7192.7584739699996</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -9495,7 +9507,7 @@
         <v>195</v>
       </c>
       <c r="B20" s="43">
-        <v>6251.3278832100004</v>
+        <v>555.51545514999998</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -9503,7 +9515,7 @@
         <v>196</v>
       </c>
       <c r="B21" s="44">
-        <v>484.15647494000001</v>
+        <v>1067.8667938200001</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -9511,7 +9523,7 @@
         <v>197</v>
       </c>
       <c r="B22" s="44">
-        <v>928.84081617000004</v>
+        <v>6629.1812545700004</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -9519,7 +9531,7 @@
         <v>198</v>
       </c>
       <c r="B23" s="44">
-        <v>4.7688800000000005E-3</v>
+        <v>588.55855565000002</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -9527,7 +9539,7 @@
         <v>199</v>
       </c>
       <c r="B24" s="44">
-        <v>510.76962545999999</v>
+        <v>757.31480059</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -9535,7 +9547,7 @@
         <v>200</v>
       </c>
       <c r="B25" s="44">
-        <v>644.35921371999996</v>
+        <v>1860.5448149700001</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -9543,7 +9555,7 @@
         <v>201</v>
       </c>
       <c r="B26" s="44">
-        <v>1610.9767362600001</v>
+        <v>1326.24926863</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -9551,7 +9563,7 @@
         <v>187</v>
       </c>
       <c r="B27" s="44">
-        <v>1114.6196868300001</v>
+        <v>1036.7040162799999</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -9559,7 +9571,7 @@
         <v>202</v>
       </c>
       <c r="B28" s="44">
-        <v>957.60056095000004</v>
+        <v>3468.9390560100001</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -9567,7 +9579,7 @@
         <v>173</v>
       </c>
       <c r="B29" s="43">
-        <v>3045.5730030099999</v>
+        <v>892.10058498000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
"Agrego emae jul26 y pobreza 1er semestre"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBC8E71-BF5A-4238-900B-3014B1CBBE25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC24659-D3E9-4A5F-A4B3-A6426478F50D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -915,7 +915,7 @@
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -982,8 +982,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="12" fillId="5" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3558,7 +3556,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -3588,10 +3586,10 @@
         <v>134.74645041349706</v>
       </c>
       <c r="C2" s="36">
-        <v>147.90228794480254</v>
+        <v>147.887593170922</v>
       </c>
       <c r="D2" s="36">
-        <v>147.05884131449477</v>
+        <v>147.18424579098183</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3602,10 +3600,10 @@
         <v>134.23236103862521</v>
       </c>
       <c r="C3" s="36">
-        <v>146.86931898530125</v>
+        <v>146.92830205978859</v>
       </c>
       <c r="D3" s="36">
-        <v>146.48052100056762</v>
+        <v>146.59760435694591</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3616,10 +3614,10 @@
         <v>150.0878942366954</v>
       </c>
       <c r="C4" s="36">
-        <v>145.97749833883569</v>
+        <v>145.94166823742799</v>
       </c>
       <c r="D4" s="36">
-        <v>145.93166785307798</v>
+        <v>146.04312469616067</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3630,10 +3628,10 @@
         <v>153.25067436662908</v>
       </c>
       <c r="C5" s="36">
-        <v>144.70807119513321</v>
+        <v>144.90155238631286</v>
       </c>
       <c r="D5" s="36">
-        <v>145.44994793136155</v>
+        <v>145.55817953783682</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3644,10 +3642,10 @@
         <v>163.51360808690507</v>
       </c>
       <c r="C6" s="36">
-        <v>144.62478893925029</v>
+        <v>144.38629711549041</v>
       </c>
       <c r="D6" s="36">
-        <v>145.0638187966789</v>
+        <v>145.1703212006199</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3658,10 +3656,10 @@
         <v>153.66209524099784</v>
       </c>
       <c r="C7" s="36">
-        <v>144.40593395794969</v>
+        <v>144.40459782140911</v>
       </c>
       <c r="D7" s="36">
-        <v>144.795120666016</v>
+        <v>144.89997168873589</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3672,10 +3670,10 @@
         <v>143.73110098180126</v>
       </c>
       <c r="C8" s="36">
-        <v>144.56971196835462</v>
+        <v>144.59024864061172</v>
       </c>
       <c r="D8" s="36">
-        <v>144.65413849762604</v>
+        <v>144.75787353356247</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3686,10 +3684,10 @@
         <v>143.6741026486049</v>
       </c>
       <c r="C9" s="36">
-        <v>145.62439225744868</v>
+        <v>145.51215513350996</v>
       </c>
       <c r="D9" s="36">
-        <v>144.6438070847106</v>
+        <v>144.74806901133289</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3700,10 +3698,10 @@
         <v>142.00773744282046</v>
       </c>
       <c r="C10" s="36">
-        <v>145.01346587648703</v>
+        <v>145.13482821110247</v>
       </c>
       <c r="D10" s="36">
-        <v>144.76293538516143</v>
+        <v>144.87009846296874</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3714,10 +3712,10 @@
         <v>141.13686329808141</v>
       </c>
       <c r="C11" s="36">
-        <v>145.13693619452528</v>
+        <v>145.1063094326301</v>
       </c>
       <c r="D11" s="36">
-        <v>145.00324154007509</v>
+        <v>145.11577537370678</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3728,10 +3726,10 @@
         <v>144.93832064073018</v>
       </c>
       <c r="C12" s="36">
-        <v>145.78761585131699</v>
+        <v>145.6975240645707</v>
       </c>
       <c r="D12" s="36">
-        <v>145.34973845890553</v>
+        <v>145.47148353465951</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3742,10 +3740,10 @@
         <v>142.59014516031914</v>
       </c>
       <c r="C13" s="36">
-        <v>146.95133257211731</v>
+        <v>147.08027784656963</v>
       </c>
       <c r="D13" s="36">
-        <v>145.7898359883429</v>
+        <v>145.92418508493483</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3756,10 +3754,10 @@
         <v>136.63265948316212</v>
       </c>
       <c r="C14" s="36">
-        <v>147.10315056347034</v>
+        <v>146.88615119206821</v>
       </c>
       <c r="D14" s="36">
-        <v>146.30916445024215</v>
+        <v>146.45744132226113</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3770,10 +3768,10 @@
         <v>132.15851633982274</v>
       </c>
       <c r="C15" s="36">
-        <v>146.83985693267059</v>
+        <v>146.91673027111494</v>
       </c>
       <c r="D15" s="36">
-        <v>146.88994972865572</v>
+        <v>147.05166637532182</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3784,10 +3782,10 @@
         <v>152.6209585590573</v>
       </c>
       <c r="C16" s="36">
-        <v>147.67109458512658</v>
+        <v>147.78747172353522</v>
       </c>
       <c r="D16" s="36">
-        <v>147.51460995597441</v>
+        <v>147.6868040657892</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3798,10 +3796,10 @@
         <v>151.94634480448738</v>
       </c>
       <c r="C17" s="36">
-        <v>147.66807814570066</v>
+        <v>147.80521427639877</v>
       </c>
       <c r="D17" s="36">
-        <v>148.16341792098223</v>
+        <v>148.34116862082203</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3812,10 +3810,10 @@
         <v>168.38920946936781</v>
       </c>
       <c r="C18" s="36">
-        <v>148.68211497089837</v>
+        <v>148.53885216159358</v>
       </c>
       <c r="D18" s="36">
-        <v>148.81064989468004</v>
+        <v>148.98730775394918</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3826,10 +3824,10 @@
         <v>161.03568546945232</v>
       </c>
       <c r="C19" s="36">
-        <v>150.26860128620675</v>
+        <v>150.30657968196169</v>
       </c>
       <c r="D19" s="36">
-        <v>149.4263530717264</v>
+        <v>149.59465378086213</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3840,10 +3838,10 @@
         <v>150.30605012391999</v>
       </c>
       <c r="C20" s="36">
-        <v>150.45415651887882</v>
+        <v>150.41811439036874</v>
       </c>
       <c r="D20" s="36">
-        <v>149.97613834878806</v>
+        <v>150.12941127019207</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3854,10 +3852,10 @@
         <v>149.25534277384111</v>
       </c>
       <c r="C21" s="36">
-        <v>150.39131093623385</v>
+        <v>150.36099655674727</v>
       </c>
       <c r="D21" s="36">
-        <v>150.42258328427556</v>
+        <v>150.5559297275577</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3868,10 +3866,10 @@
         <v>146.38655965775385</v>
       </c>
       <c r="C22" s="36">
-        <v>151.21376013876639</v>
+        <v>151.27260879655293</v>
       </c>
       <c r="D22" s="36">
-        <v>150.72715127054451</v>
+        <v>150.83847878949234</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3882,10 +3880,10 @@
         <v>149.38594966601454</v>
       </c>
       <c r="C23" s="36">
-        <v>151.69328476469425</v>
+        <v>151.55523864503513</v>
       </c>
       <c r="D23" s="36">
-        <v>150.85914085952476</v>
+        <v>150.94963663491373</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -3896,10 +3894,10 @@
         <v>151.92604285202697</v>
       </c>
       <c r="C24" s="36">
-        <v>152.61081737406121</v>
+        <v>152.67042574504046</v>
       </c>
       <c r="D24" s="36">
-        <v>150.79269365352215</v>
+        <v>150.86658814918212</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3910,10 +3908,10 @@
         <v>146.78338490922451</v>
       </c>
       <c r="C25" s="36">
-        <v>152.23047843206538</v>
+        <v>152.30832124827532</v>
       </c>
       <c r="D25" s="36">
-        <v>150.51491752532093</v>
+        <v>150.57871769261894</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -3924,10 +3922,10 @@
         <v>142.74091260617223</v>
       </c>
       <c r="C26" s="36">
-        <v>150.97432403194165</v>
+        <v>150.81647854773971</v>
       </c>
       <c r="D26" s="36">
-        <v>150.03080673561695</v>
+        <v>150.09189614428379</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3938,10 +3936,10 @@
         <v>138.81804035165743</v>
       </c>
       <c r="C27" s="36">
-        <v>152.21496614021012</v>
+        <v>152.31300321897666</v>
       </c>
       <c r="D27" s="36">
-        <v>149.3624332264886</v>
+        <v>149.42780353006791</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3952,10 +3950,10 @@
         <v>155.85731953576973</v>
       </c>
       <c r="C28" s="36">
-        <v>151.54850660607454</v>
+        <v>151.64408973312376</v>
       </c>
       <c r="D28" s="36">
-        <v>148.54828673930285</v>
+        <v>148.62288336710569</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3966,10 +3964,10 @@
         <v>151.52454398394343</v>
       </c>
       <c r="C29" s="36">
-        <v>146.80644414143845</v>
+        <v>146.84457724330429</v>
       </c>
       <c r="D29" s="36">
-        <v>147.63523092998457</v>
+        <v>147.72179013281686</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -3980,10 +3978,10 @@
         <v>159.5666923779167</v>
       </c>
       <c r="C30" s="36">
-        <v>144.58761676999234</v>
+        <v>144.54354601439613</v>
       </c>
       <c r="D30" s="36">
-        <v>146.67848734799458</v>
+        <v>146.77741192020974</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3994,10 +3992,10 @@
         <v>151.12576323345522</v>
       </c>
       <c r="C31" s="36">
-        <v>143.27264246575626</v>
+        <v>143.27773048362042</v>
       </c>
       <c r="D31" s="36">
-        <v>145.73584383725961</v>
+        <v>145.84534542519717</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -4008,10 +4006,10 @@
         <v>145.96352443000461</v>
       </c>
       <c r="C32" s="36">
-        <v>143.59456149815151</v>
+        <v>143.47840462948142</v>
       </c>
       <c r="D32" s="36">
-        <v>144.85986468982435</v>
+        <v>144.97734669052628</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -4022,10 +4020,10 @@
         <v>146.76596003413968</v>
       </c>
       <c r="C33" s="36">
-        <v>146.54647689029972</v>
+        <v>146.6859767064804</v>
       </c>
       <c r="D33" s="36">
-        <v>144.09839390385193</v>
+        <v>144.22053177465861</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -4036,10 +4034,10 @@
         <v>137.746569718648</v>
       </c>
       <c r="C34" s="36">
-        <v>143.13178589235872</v>
+        <v>143.06658186535478</v>
       </c>
       <c r="D34" s="36">
-        <v>143.48526623050319</v>
+        <v>143.60889862301462</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -4050,10 +4048,10 @@
         <v>142.84327598456761</v>
       </c>
       <c r="C35" s="36">
-        <v>143.55929161700038</v>
+        <v>143.48138739235543</v>
       </c>
       <c r="D35" s="36">
-        <v>143.03626587801961</v>
+        <v>143.15929618672342</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -4064,10 +4062,10 @@
         <v>140.59240732533567</v>
       </c>
       <c r="C36" s="36">
-        <v>141.61755948831191</v>
+        <v>141.69639549597727</v>
       </c>
       <c r="D36" s="36">
-        <v>142.75240421627376</v>
+        <v>142.87430846205777</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -4078,10 +4076,10 @@
         <v>136.25161596905636</v>
       </c>
       <c r="C37" s="36">
-        <v>141.94245053564785</v>
+        <v>141.94845478524581</v>
       </c>
       <c r="D37" s="36">
-        <v>142.62030929088488</v>
+        <v>142.74117962526864</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -4092,10 +4090,10 @@
         <v>134.5362398566958</v>
       </c>
       <c r="C38" s="36">
-        <v>141.42634449054745</v>
+        <v>141.3468168733616</v>
       </c>
       <c r="D38" s="36">
-        <v>142.61157661917866</v>
+        <v>142.732433256577</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -4106,10 +4104,10 @@
         <v>132.26788861273661</v>
       </c>
       <c r="C39" s="36">
-        <v>143.72785091696355</v>
+        <v>143.75217660409459</v>
       </c>
       <c r="D39" s="36">
-        <v>142.68844745241501</v>
+        <v>142.81074564073205</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -4120,10 +4118,10 @@
         <v>144.96325495574916</v>
       </c>
       <c r="C40" s="36">
-        <v>142.33640443007181</v>
+        <v>142.33422947253123</v>
       </c>
       <c r="D40" s="36">
-        <v>142.80929312695918</v>
+        <v>142.93379910428564</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -4134,10 +4132,10 @@
         <v>149.91622140352271</v>
       </c>
       <c r="C41" s="36">
-        <v>142.63217066739119</v>
+        <v>142.53281997752035</v>
       </c>
       <c r="D41" s="36">
-        <v>142.92899490596105</v>
+        <v>143.05560431140691</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4148,10 +4146,10 @@
         <v>164.1356990759204</v>
       </c>
       <c r="C42" s="36">
-        <v>144.85176283668281</v>
+        <v>145.02221705182123</v>
       </c>
       <c r="D42" s="36">
-        <v>143.00611711109545</v>
+        <v>143.13512794092233</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -4162,10 +4160,10 @@
         <v>150.85897174113128</v>
       </c>
       <c r="C43" s="36">
-        <v>144.04490409998212</v>
+        <v>143.99907879678125</v>
       </c>
       <c r="D43" s="36">
-        <v>143.00568802760029</v>
+        <v>143.13830309304473</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -4176,10 +4174,10 @@
         <v>146.77702964007034</v>
       </c>
       <c r="C44" s="36">
-        <v>145.82192292861072</v>
+        <v>145.82398411185972</v>
       </c>
       <c r="D44" s="36">
-        <v>142.90114762770563</v>
+        <v>143.03890653914942</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -4190,10 +4188,10 @@
         <v>141.27693468084036</v>
       </c>
       <c r="C45" s="36">
-        <v>144.77374425103372</v>
+        <v>144.88827244423732</v>
       </c>
       <c r="D45" s="36">
-        <v>142.67645193678277</v>
+        <v>142.8211067832097</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -4204,10 +4202,10 @@
         <v>134.87706647993653</v>
       </c>
       <c r="C46" s="36">
-        <v>140.52870612823389</v>
+        <v>140.44516327540947</v>
       </c>
       <c r="D46" s="36">
-        <v>142.32683422868618</v>
+        <v>142.47998169196538</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -4218,10 +4216,10 @@
         <v>141.63933661701381</v>
       </c>
       <c r="C47" s="36">
-        <v>143.75161347511875</v>
+        <v>143.79187156014729</v>
       </c>
       <c r="D47" s="36">
-        <v>141.85824620693592</v>
+        <v>142.02103631457587</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -4232,10 +4230,10 @@
         <v>137.77182966933145</v>
       </c>
       <c r="C48" s="36">
-        <v>140.81021564190533</v>
+        <v>140.86717496872228</v>
       </c>
       <c r="D48" s="36">
-        <v>141.28726807080514</v>
+        <v>141.46025660037981</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -4246,10 +4244,10 @@
         <v>135.76515452763502</v>
       </c>
       <c r="C49" s="36">
-        <v>140.07998791005343</v>
+        <v>139.98182267819982</v>
       </c>
       <c r="D49" s="36">
-        <v>140.64135515964173</v>
+        <v>140.82619215378955</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -4260,10 +4258,10 @@
         <v>133.89108608957241</v>
       </c>
       <c r="C50" s="36">
-        <v>140.92554601700547</v>
+        <v>141.02722801226969</v>
       </c>
       <c r="D50" s="36">
-        <v>139.9508919074238</v>
+        <v>140.14848095835015</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -4274,10 +4272,10 @@
         <v>128.97363874659823</v>
       </c>
       <c r="C51" s="36">
-        <v>139.58431341498277</v>
+        <v>139.69021424767496</v>
       </c>
       <c r="D51" s="36">
-        <v>139.24950149986981</v>
+        <v>139.45941224630388</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -4288,10 +4286,10 @@
         <v>128.21106074025667</v>
       </c>
       <c r="C52" s="36">
-        <v>126.02034936546131</v>
+        <v>125.81858245148825</v>
       </c>
       <c r="D52" s="36">
-        <v>138.57159350028013</v>
+        <v>138.79134071814818</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -4302,10 +4300,10 @@
         <v>113.29503444580156</v>
       </c>
       <c r="C53" s="36">
-        <v>106.05639981841499</v>
+        <v>106.13633643303258</v>
       </c>
       <c r="D53" s="36">
-        <v>137.95177444201141</v>
+        <v>138.17765563745647</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -4316,10 +4314,10 @@
         <v>131.02956919734916</v>
       </c>
       <c r="C54" s="36">
-        <v>117.26625454147219</v>
+        <v>117.33435908923668</v>
       </c>
       <c r="D54" s="36">
-        <v>137.42336915504214</v>
+        <v>137.65025481007604</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -4330,10 +4328,10 @@
         <v>132.52196526648777</v>
       </c>
       <c r="C55" s="36">
-        <v>124.35972004671306</v>
+        <v>124.18693388507192</v>
       </c>
       <c r="D55" s="36">
-        <v>137.01191055029554</v>
+        <v>137.23479177004401</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -4344,10 +4342,10 @@
         <v>127.46368946979405</v>
       </c>
       <c r="C56" s="36">
-        <v>126.14854476042942</v>
+        <v>126.39019367275476</v>
       </c>
       <c r="D56" s="36">
-        <v>136.73449987129194</v>
+        <v>136.94973561250913</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -4358,10 +4356,10 @@
         <v>125.18389375984655</v>
       </c>
       <c r="C57" s="36">
-        <v>128.83372679932165</v>
+        <v>128.75881140508946</v>
       </c>
       <c r="D57" s="36">
-        <v>136.60088049432886</v>
+        <v>136.80700286623241</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -4372,10 +4370,10 @@
         <v>127.17507609335286</v>
       </c>
       <c r="C58" s="36">
-        <v>130.76173160851343</v>
+        <v>130.59946668347575</v>
       </c>
       <c r="D58" s="36">
-        <v>136.61209476684212</v>
+        <v>136.80878515998577</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -4386,10 +4384,10 @@
         <v>131.34550189452798</v>
       </c>
       <c r="C59" s="36">
-        <v>133.35013477038626</v>
+        <v>133.44789400258284</v>
       </c>
       <c r="D59" s="36">
-        <v>136.76269563502817</v>
+        <v>136.94949960911188</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -4400,10 +4398,10 @@
         <v>132.06865525299673</v>
       </c>
       <c r="C60" s="36">
-        <v>134.79827594761082</v>
+        <v>134.68442065803782</v>
       </c>
       <c r="D60" s="36">
-        <v>137.03990402352059</v>
+        <v>137.21612637755678</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -4414,10 +4412,10 @@
         <v>133.85436559460618</v>
       </c>
       <c r="C61" s="36">
-        <v>136.90853992586401</v>
+        <v>136.93909650977974</v>
       </c>
       <c r="D61" s="36">
-        <v>137.42718773237806</v>
+        <v>137.5917736470571</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -4428,10 +4426,10 @@
         <v>131.52153739731895</v>
       </c>
       <c r="C62" s="36">
-        <v>139.85869931136128</v>
+        <v>139.82109534931803</v>
       </c>
       <c r="D62" s="36">
-        <v>137.90773055216602</v>
+        <v>138.05920860504034</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -4442,10 +4440,10 @@
         <v>126.23926696836419</v>
       </c>
       <c r="C63" s="36">
-        <v>138.27778724368201</v>
+        <v>138.39777937737929</v>
       </c>
       <c r="D63" s="36">
-        <v>138.46922791775205</v>
+        <v>138.60608473842595</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -4456,10 +4454,10 @@
         <v>145.9569001036472</v>
       </c>
       <c r="C64" s="36">
-        <v>140.94283751059339</v>
+        <v>140.84149978974523</v>
       </c>
       <c r="D64" s="36">
-        <v>139.1015222090131</v>
+        <v>139.22218597404691</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -4470,10 +4468,10 @@
         <v>147.28084401875961</v>
       </c>
       <c r="C65" s="36">
-        <v>139.42174873428777</v>
+        <v>139.54243216964221</v>
       </c>
       <c r="D65" s="36">
-        <v>139.80063611380118</v>
+        <v>139.90346864151056</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -4484,10 +4482,10 @@
         <v>151.16932233874826</v>
       </c>
       <c r="C66" s="36">
-        <v>138.92350185503292</v>
+        <v>138.90768268428616</v>
       </c>
       <c r="D66" s="36">
-        <v>140.56490592146289</v>
+        <v>140.65036155695188</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -4498,10 +4496,10 @@
         <v>148.97961710841247</v>
       </c>
       <c r="C67" s="36">
-        <v>141.54410781899168</v>
+        <v>141.41079892250298</v>
       </c>
       <c r="D67" s="36">
-        <v>141.39166062844572</v>
+        <v>141.46156634208171</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -4512,10 +4510,10 @@
         <v>142.42591306035814</v>
       </c>
       <c r="C68" s="36">
-        <v>141.35346521561027</v>
+        <v>141.54080839761772</v>
       </c>
       <c r="D68" s="36">
-        <v>142.28165460957507</v>
+        <v>142.33910344031071</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -4526,10 +4524,10 @@
         <v>140.97494072777735</v>
       </c>
       <c r="C69" s="36">
-        <v>143.29318922352883</v>
+        <v>143.14909480065771</v>
       </c>
       <c r="D69" s="36">
-        <v>143.23502605857846</v>
+        <v>143.28428297807804</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -4537,13 +4535,13 @@
         <v>44440</v>
       </c>
       <c r="B70" s="17">
-        <v>141.29608909028411</v>
+        <v>141.29608909028414</v>
       </c>
       <c r="C70" s="36">
-        <v>144.12507279457796</v>
+        <v>144.13657482152971</v>
       </c>
       <c r="D70" s="36">
-        <v>144.24592259774104</v>
+        <v>144.29144951896745</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -4554,10 +4552,10 @@
         <v>139.51475869967891</v>
       </c>
       <c r="C71" s="36">
-        <v>143.32018242264803</v>
+        <v>143.33782925992301</v>
       </c>
       <c r="D71" s="36">
-        <v>145.30255603451579</v>
+        <v>145.34791598208167</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -4568,10 +4566,10 @@
         <v>143.75187761888859</v>
       </c>
       <c r="C72" s="36">
-        <v>145.6282008947839</v>
+        <v>145.38932717790323</v>
       </c>
       <c r="D72" s="36">
-        <v>146.38014447859447</v>
+        <v>146.42801883635101</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -4582,10 +4580,10 @@
         <v>147.2298783181341</v>
       </c>
       <c r="C73" s="36">
-        <v>149.65215293879575</v>
+        <v>149.86602325129434</v>
       </c>
       <c r="D73" s="36">
-        <v>147.44080755534532</v>
+        <v>147.49294737804229</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -4593,13 +4591,13 @@
         <v>44562</v>
       </c>
       <c r="B74" s="17">
-        <v>139.6379616122818</v>
+        <v>139.63796161228177</v>
       </c>
       <c r="C74" s="36">
-        <v>148.50300074015578</v>
+        <v>148.29249185627833</v>
       </c>
       <c r="D74" s="36">
-        <v>148.4404600410748</v>
+        <v>148.49659959515188</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -4610,10 +4608,10 @@
         <v>137.84951352507593</v>
       </c>
       <c r="C75" s="36">
-        <v>150.71219600987763</v>
+        <v>150.84322740553762</v>
       </c>
       <c r="D75" s="36">
-        <v>149.33271238306372</v>
+        <v>149.3935263572624</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -4621,13 +4619,13 @@
         <v>44621</v>
       </c>
       <c r="B76" s="17">
-        <v>153.93085079425231</v>
+        <v>153.93085079425236</v>
       </c>
       <c r="C76" s="36">
-        <v>150.36649250775957</v>
+        <v>150.46306825037135</v>
       </c>
       <c r="D76" s="36">
-        <v>150.07881778771394</v>
+        <v>150.14407504825786</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -4635,13 +4633,13 @@
         <v>44652</v>
       </c>
       <c r="B77" s="17">
-        <v>157.66169217344401</v>
+        <v>157.66169217344412</v>
       </c>
       <c r="C77" s="36">
-        <v>152.26721240793535</v>
+        <v>152.37835769985364</v>
       </c>
       <c r="D77" s="36">
-        <v>150.651089556285</v>
+        <v>150.71992372617987</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -4649,13 +4647,13 @@
         <v>44682</v>
       </c>
       <c r="B78" s="17">
-        <v>164.68936311408291</v>
+        <v>164.68936311408294</v>
       </c>
       <c r="C78" s="36">
-        <v>152.22665108010588</v>
+        <v>152.11179883083747</v>
       </c>
       <c r="D78" s="36">
-        <v>151.03332176495991</v>
+        <v>151.10432895334196</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -4663,13 +4661,13 @@
         <v>44713</v>
       </c>
       <c r="B79" s="17">
-        <v>161.45483428121702</v>
+        <v>161.45483428121688</v>
       </c>
       <c r="C79" s="36">
-        <v>154.32065688488396</v>
+        <v>154.27426044152489</v>
       </c>
       <c r="D79" s="36">
-        <v>151.22201815253945</v>
+        <v>151.29473597165716</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -4677,13 +4675,13 @@
         <v>44743</v>
       </c>
       <c r="B80" s="17">
-        <v>152.4453874358741</v>
+        <v>152.44538743587361</v>
       </c>
       <c r="C80" s="36">
-        <v>152.52038638813951</v>
+        <v>152.61462497882655</v>
       </c>
       <c r="D80" s="36">
-        <v>151.23059877801032</v>
+        <v>151.30495808494919</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -4691,13 +4689,13 @@
         <v>44774</v>
       </c>
       <c r="B81" s="17">
-        <v>151.46573891606729</v>
+        <v>151.4657389160671</v>
       </c>
       <c r="C81" s="36">
-        <v>151.65878749519123</v>
+        <v>151.58821866488825</v>
       </c>
       <c r="D81" s="36">
-        <v>151.08612942118208</v>
+        <v>151.16227687431078</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -4705,13 +4703,13 @@
         <v>44805</v>
       </c>
       <c r="B82" s="17">
-        <v>149.17434970526307</v>
+        <v>149.17434970526381</v>
       </c>
       <c r="C82" s="36">
-        <v>150.70875085496451</v>
+        <v>150.76162166948612</v>
       </c>
       <c r="D82" s="36">
-        <v>150.82457670878878</v>
+        <v>150.90298114328121</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -4719,13 +4717,13 @@
         <v>44835</v>
       </c>
       <c r="B83" s="17">
-        <v>146.55439616164352</v>
+        <v>146.55439616164583</v>
       </c>
       <c r="C83" s="36">
-        <v>149.06554743419156</v>
+        <v>148.98975163637644</v>
       </c>
       <c r="D83" s="36">
-        <v>150.48557863738</v>
+        <v>150.5667253111763</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -4733,13 +4731,13 @@
         <v>44866</v>
       </c>
       <c r="B84" s="17">
-        <v>148.03049492949961</v>
+        <v>148.03049492950063</v>
       </c>
       <c r="C84" s="36">
-        <v>148.29221401437047</v>
+        <v>148.14110524181046</v>
       </c>
       <c r="D84" s="36">
-        <v>150.10659984539819</v>
+        <v>150.19158339292829</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -4747,13 +4745,13 @@
         <v>44896</v>
       </c>
       <c r="B85" s="17">
-        <v>146.18080633804541</v>
+        <v>146.1808063380422</v>
       </c>
       <c r="C85" s="36">
-        <v>148.43349371359295</v>
+        <v>148.61686289556908</v>
       </c>
       <c r="D85" s="36">
-        <v>149.72034836077549</v>
+        <v>149.81028571328625</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -4761,13 +4759,13 @@
         <v>44927</v>
       </c>
       <c r="B86" s="17">
-        <v>143.03462349514643</v>
+        <v>143.03462349513615</v>
       </c>
       <c r="C86" s="36">
-        <v>149.92114342631578</v>
+        <v>149.53638197645233</v>
       </c>
       <c r="D86" s="36">
-        <v>149.34922137615646</v>
+        <v>149.44498568929976</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -4775,13 +4773,13 @@
         <v>44958</v>
       </c>
       <c r="B87" s="17">
-        <v>137.26646276487918</v>
+        <v>137.26646276487486</v>
       </c>
       <c r="C87" s="36">
-        <v>150.10029003096659</v>
+        <v>150.2042105117583</v>
       </c>
       <c r="D87" s="36">
-        <v>149.00211604628635</v>
+        <v>149.10405134691487</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -4789,13 +4787,13 @@
         <v>44986</v>
       </c>
       <c r="B88" s="17">
-        <v>155.06501366860087</v>
+        <v>155.06501366861548</v>
       </c>
       <c r="C88" s="36">
-        <v>150.75256289433395</v>
+        <v>151.03523442820438</v>
       </c>
       <c r="D88" s="36">
-        <v>148.67363087150412</v>
+        <v>148.78082538946359</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -4803,13 +4801,13 @@
         <v>45017</v>
       </c>
       <c r="B89" s="17">
-        <v>150.05952685002168</v>
+        <v>150.05952685006818</v>
       </c>
       <c r="C89" s="36">
-        <v>147.53224583499846</v>
+        <v>147.54192655097015</v>
       </c>
       <c r="D89" s="36">
-        <v>148.34803699709209</v>
+        <v>148.45963620181746</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -4817,13 +4815,13 @@
         <v>45047</v>
       </c>
       <c r="B90" s="17">
-        <v>153.81085419208719</v>
+        <v>153.81085419210677</v>
       </c>
       <c r="C90" s="36">
-        <v>145.62328742845165</v>
+        <v>145.60872138350896</v>
       </c>
       <c r="D90" s="36">
-        <v>148.0018911303971</v>
+        <v>148.11829972716782</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -4831,13 +4829,13 @@
         <v>45078</v>
       </c>
       <c r="B91" s="17">
-        <v>152.59547604983808</v>
+        <v>152.59547604977197</v>
       </c>
       <c r="C91" s="36">
-        <v>146.08926594642224</v>
+        <v>145.97619826349731</v>
       </c>
       <c r="D91" s="36">
-        <v>147.61471669119589</v>
+        <v>147.7366269547274</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -4845,13 +4843,13 @@
         <v>45108</v>
       </c>
       <c r="B92" s="17">
-        <v>150.20312548746972</v>
+        <v>150.20312548725906</v>
       </c>
       <c r="C92" s="36">
-        <v>148.6911839315234</v>
+        <v>148.70852732358321</v>
       </c>
       <c r="D92" s="36">
-        <v>147.17511504295197</v>
+        <v>147.30320557656174</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -4859,13 +4857,13 @@
         <v>45139</v>
       </c>
       <c r="B93" s="17">
-        <v>151.92217936039572</v>
+        <v>151.92217936030693</v>
       </c>
       <c r="C93" s="36">
-        <v>150.0285645140801</v>
+        <v>150.07156029479671</v>
       </c>
       <c r="D93" s="36">
-        <v>146.68020263880157</v>
+        <v>146.81458781623891</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -4873,13 +4871,13 @@
         <v>45170</v>
       </c>
       <c r="B94" s="17">
-        <v>148.41237963196167</v>
+        <v>148.41237963226115</v>
       </c>
       <c r="C94" s="36">
-        <v>149.64368007725099</v>
+        <v>149.70616184019144</v>
       </c>
       <c r="D94" s="36">
-        <v>146.14050006800522</v>
+        <v>146.2805573138676</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -4887,13 +4885,13 @@
         <v>45200</v>
       </c>
       <c r="B95" s="17">
-        <v>147.51381302893859</v>
+        <v>147.5138130298927</v>
       </c>
       <c r="C95" s="36">
-        <v>148.00946878449926</v>
+        <v>147.83107824820434</v>
       </c>
       <c r="D95" s="36">
-        <v>145.57967263807711</v>
+        <v>145.72444581327431</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -4901,13 +4899,13 @@
         <v>45231</v>
       </c>
       <c r="B96" s="17">
-        <v>146.36635231658468</v>
+        <v>146.36635231698688</v>
       </c>
       <c r="C96" s="36">
-        <v>146.35986201157135</v>
+        <v>146.38154070926913</v>
       </c>
       <c r="D96" s="36">
-        <v>145.02944531059569</v>
+        <v>145.17812854123</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -4915,13 +4913,13 @@
         <v>45261</v>
       </c>
       <c r="B97" s="17">
-        <v>139.342627273609</v>
+        <v>139.34262727225266</v>
       </c>
       <c r="C97" s="36">
-        <v>142.8408797734873</v>
+        <v>142.99089316291239</v>
       </c>
       <c r="D97" s="36">
-        <v>144.53417943799141</v>
+        <v>144.68622332253389</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -4929,13 +4927,13 @@
         <v>45292</v>
       </c>
       <c r="B98" s="17">
-        <v>137.37335131476613</v>
+        <v>137.3733513104446</v>
       </c>
       <c r="C98" s="36">
-        <v>143.50372627874964</v>
+        <v>143.05741568961781</v>
       </c>
       <c r="D98" s="36">
-        <v>144.14240026401174</v>
+        <v>144.2976417090826</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4943,13 +4941,13 @@
         <v>45323</v>
       </c>
       <c r="B99" s="17">
-        <v>133.46450585818494</v>
+        <v>133.4645058563633</v>
       </c>
       <c r="C99" s="36">
-        <v>143.73405745303077</v>
+        <v>143.8710263395235</v>
       </c>
       <c r="D99" s="36">
-        <v>143.90035667692231</v>
+        <v>144.05602406994728</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4957,13 +4955,13 @@
         <v>45352</v>
       </c>
       <c r="B100" s="17">
-        <v>142.39572369405857</v>
+        <v>142.39572370020173</v>
       </c>
       <c r="C100" s="36">
-        <v>142.0898066454663</v>
+        <v>142.33397234616913</v>
       </c>
       <c r="D100" s="36">
-        <v>143.84698353493195</v>
+        <v>143.99888093803492</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -4971,13 +4969,13 @@
         <v>45383</v>
       </c>
       <c r="B101" s="17">
-        <v>147.25689957052242</v>
+        <v>147.25689959009534</v>
       </c>
       <c r="C101" s="36">
-        <v>141.12508437171982</v>
+        <v>141.09484926770605</v>
       </c>
       <c r="D101" s="36">
-        <v>144.00290416304108</v>
+        <v>144.14905087201089</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -4985,13 +4983,13 @@
         <v>45413</v>
       </c>
       <c r="B102" s="17">
-        <v>156.76909867816687</v>
+        <v>156.76909868641758</v>
       </c>
       <c r="C102" s="36">
-        <v>142.83832491106693</v>
+        <v>143.12009217669834</v>
       </c>
       <c r="D102" s="36">
-        <v>144.36812819412728</v>
+        <v>144.50860899177152</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -4999,13 +4997,13 @@
         <v>45444</v>
       </c>
       <c r="B103" s="17">
-        <v>147.35712225489846</v>
+        <v>147.35712222707485</v>
       </c>
       <c r="C103" s="36">
-        <v>143.68907555762658</v>
+        <v>143.33433573160545</v>
       </c>
       <c r="D103" s="36">
-        <v>144.92532565270611</v>
+        <v>145.06136657110196</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -5013,13 +5011,13 @@
         <v>45474</v>
       </c>
       <c r="B104" s="17">
-        <v>149.65170282067913</v>
+        <v>149.65170273202926</v>
       </c>
       <c r="C104" s="36">
-        <v>147.28415957594882</v>
+        <v>147.24503227828828</v>
       </c>
       <c r="D104" s="36">
-        <v>145.63964072356882</v>
+        <v>145.77501250467688</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -5027,13 +5025,13 @@
         <v>45505</v>
       </c>
       <c r="B105" s="17">
-        <v>147.28124861080667</v>
+        <v>147.28124857343758</v>
       </c>
       <c r="C105" s="36">
-        <v>147.82949220892567</v>
+        <v>147.99748002160811</v>
       </c>
       <c r="D105" s="36">
-        <v>146.46314634054664</v>
+        <v>146.60376991264943</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -5041,13 +5039,13 @@
         <v>45536</v>
       </c>
       <c r="B106" s="17">
-        <v>144.79669856581739</v>
+        <v>144.79669869183633</v>
       </c>
       <c r="C106" s="36">
-        <v>147.86734414916225</v>
+        <v>147.82869498844457</v>
       </c>
       <c r="D106" s="36">
-        <v>147.34307891115623</v>
+        <v>147.495321779401</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -5055,13 +5053,13 @@
         <v>45566</v>
       </c>
       <c r="B107" s="17">
-        <v>148.10394079332772</v>
+        <v>148.10394119484172</v>
       </c>
       <c r="C107" s="36">
-        <v>149.07724609103079</v>
+        <v>149.10719503402422</v>
       </c>
       <c r="D107" s="36">
-        <v>148.22246905613449</v>
+        <v>148.39291446354324</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -5069,13 +5067,13 @@
         <v>45597</v>
       </c>
       <c r="B108" s="17">
-        <v>148.17872904548861</v>
+        <v>148.17872921474091</v>
       </c>
       <c r="C108" s="36">
-        <v>150.80674041817159</v>
+        <v>150.87021962285306</v>
       </c>
       <c r="D108" s="36">
-        <v>149.05295938117266</v>
+        <v>149.24534324319538</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -5083,13 +5081,13 @@
         <v>45627</v>
       </c>
       <c r="B109" s="17">
-        <v>148.67761660915863</v>
+        <v>148.67761603839233</v>
       </c>
       <c r="C109" s="36">
-        <v>151.46158068205571</v>
+        <v>151.44632488532656</v>
       </c>
       <c r="D109" s="36">
-        <v>149.80008623128035</v>
+        <v>150.01368489830435</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -5097,13 +5095,13 @@
         <v>45658</v>
       </c>
       <c r="B110" s="17">
-        <v>146.49668450002147</v>
+        <v>146.49668268147974</v>
       </c>
       <c r="C110" s="36">
-        <v>151.9028548224955</v>
+        <v>151.55095881861351</v>
       </c>
       <c r="D110" s="36">
-        <v>150.44087661321521</v>
+        <v>150.67135330325397</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -5111,13 +5109,13 @@
         <v>45689</v>
       </c>
       <c r="B111" s="17">
-        <v>141.40461989508793</v>
+        <v>141.40461912850864</v>
       </c>
       <c r="C111" s="36">
-        <v>153.49352013447819</v>
+        <v>153.4167608129367</v>
       </c>
       <c r="D111" s="36">
-        <v>150.96654691826183</v>
+        <v>151.20702149198854</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -5125,13 +5123,13 @@
         <v>45717</v>
       </c>
       <c r="B112" s="17">
-        <v>150.61008323211774</v>
+        <v>150.61008581723874</v>
       </c>
       <c r="C112" s="36">
-        <v>149.31840483832218</v>
+        <v>149.45568731032341</v>
       </c>
       <c r="D112" s="36">
-        <v>151.38172496348201</v>
+        <v>151.62431183635744</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -5139,13 +5137,13 @@
         <v>45748</v>
       </c>
       <c r="B113" s="17">
-        <v>158.93908114668073</v>
+        <v>158.93908938324</v>
       </c>
       <c r="C113" s="36">
-        <v>152.35852404350794</v>
+        <v>152.50837254398098</v>
       </c>
       <c r="D113" s="36">
-        <v>151.70088729461301</v>
+        <v>151.93880694603604</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -5153,13 +5151,13 @@
         <v>45778</v>
       </c>
       <c r="B114" s="17">
-        <v>165.07455171005421</v>
+        <v>165.07455518205356</v>
       </c>
       <c r="C114" s="36">
-        <v>152.12964111898245</v>
+        <v>152.46318120030611</v>
       </c>
       <c r="D114" s="36">
-        <v>151.94658597568645</v>
+        <v>152.17733722152286</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -5167,13 +5165,13 @@
         <v>45809</v>
       </c>
       <c r="B115" s="17">
-        <v>156.78921353289212</v>
+        <v>156.78920182433359</v>
       </c>
       <c r="C115" s="36">
-        <v>151.50751953044457</v>
+        <v>150.97359110411981</v>
       </c>
       <c r="D115" s="36">
-        <v>152.14393461496158</v>
+        <v>152.36757090044856</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -5181,13 +5179,13 @@
         <v>45839</v>
       </c>
       <c r="B116" s="17">
-        <v>153.77120720937</v>
+        <v>153.77116990425543</v>
       </c>
       <c r="C116" s="36">
-        <v>151.354343475533</v>
+        <v>151.54206663366895</v>
       </c>
       <c r="D116" s="36">
-        <v>152.31655807533912</v>
+        <v>152.53522842125278</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -5195,13 +5193,13 @@
         <v>45870</v>
       </c>
       <c r="B117" s="17">
-        <v>150.37620998417583</v>
+        <v>150.37619425875818</v>
       </c>
       <c r="C117" s="36">
-        <v>152.36783814947248</v>
+        <v>152.4776457529625</v>
       </c>
       <c r="D117" s="36">
-        <v>152.485181818429</v>
+        <v>152.70073407082987</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -5209,13 +5207,13 @@
         <v>45901</v>
       </c>
       <c r="B118" s="17">
-        <v>151.7041464938178</v>
+        <v>151.70419952434997</v>
       </c>
       <c r="C118" s="36">
-        <v>153.40609674320959</v>
+        <v>153.22896887402936</v>
       </c>
       <c r="D118" s="36">
-        <v>152.66272535633675</v>
+        <v>152.87914364745151</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -5223,13 +5221,13 @@
         <v>45931</v>
       </c>
       <c r="B119" s="17">
-        <v>152.83388431255179</v>
+        <v>152.83405327528675</v>
       </c>
       <c r="C119" s="36">
-        <v>153.10436298931441</v>
+        <v>153.2613988120184</v>
       </c>
       <c r="D119" s="36">
-        <v>152.85582558966763</v>
+        <v>153.0806149505581</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -5237,13 +5235,13 @@
         <v>45962</v>
       </c>
       <c r="B120" s="17">
-        <v>147.96980447689901</v>
+        <v>147.96987570063345</v>
       </c>
       <c r="C120" s="36">
-        <v>152.98368629623431</v>
+        <v>152.95402275714397</v>
       </c>
       <c r="D120" s="36">
-        <v>153.06910313427898</v>
+        <v>153.31088219407724</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -5251,13 +5249,13 @@
         <v>45992</v>
       </c>
       <c r="B121" s="17">
-        <v>153.85251211265549</v>
+        <v>153.85227192618612</v>
       </c>
       <c r="C121" s="36">
-        <v>155.89520740777738</v>
+        <v>155.98934499695974</v>
       </c>
       <c r="D121" s="36">
-        <v>153.30538384870047</v>
+        <v>153.57304585496371</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -5265,13 +5263,13 @@
         <v>46023</v>
       </c>
       <c r="B122" s="17">
-        <v>149.43188619926431</v>
+        <v>149.48602043206023</v>
       </c>
       <c r="C122" s="36">
-        <v>156.36605874815257</v>
+        <v>155.98570837693899</v>
       </c>
       <c r="D122" s="36">
-        <v>153.56717850732065</v>
+        <v>153.86286991133275</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -5279,13 +5277,13 @@
         <v>46054</v>
       </c>
       <c r="B123" s="17">
-        <v>139.3365199989212</v>
+        <v>139.34303476491058</v>
       </c>
       <c r="C123" s="36">
-        <v>152.47861532335506</v>
+        <v>152.58281982593593</v>
       </c>
       <c r="D123" s="36">
-        <v>153.8599087710904</v>
+        <v>154.17353803121014</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
@@ -5293,13 +5291,13 @@
         <v>46082</v>
       </c>
       <c r="B124" s="17">
-        <v>159.9499096193297</v>
+        <v>160.23744803364747</v>
       </c>
       <c r="C124" s="36">
-        <v>156.4698201506535</v>
+        <v>156.73695664033295</v>
       </c>
       <c r="D124" s="36">
-        <v>154.18637754509663</v>
+        <v>154.49731357422957</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
@@ -5307,13 +5305,13 @@
         <v>46113</v>
       </c>
       <c r="B125" s="17">
-        <v>161.71805294443547</v>
+        <v>162.30299655822449</v>
       </c>
       <c r="C125" s="36">
-        <v>153.90332453400006</v>
+        <v>154.60965986576048</v>
       </c>
       <c r="D125" s="36">
-        <v>154.54371532399702</v>
+        <v>154.8201721631755</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
@@ -5321,27 +5319,41 @@
         <v>46143</v>
       </c>
       <c r="B126" s="17">
-        <v>165.66808413621425</v>
+        <v>166.26832998733488</v>
       </c>
       <c r="C126" s="36">
-        <v>152.96249448451684</v>
+        <v>153.70189679546644</v>
       </c>
       <c r="D126" s="36">
-        <v>154.92890282828878</v>
+        <v>155.13932443072952</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
         <v>46174</v>
       </c>
-      <c r="B127" s="40">
-        <v>161.01331908191355</v>
-      </c>
-      <c r="C127" s="41">
-        <v>154.1172638221334</v>
-      </c>
-      <c r="D127" s="41">
-        <v>155.31027391562463</v>
+      <c r="B127" s="17">
+        <v>161.70418903034249</v>
+      </c>
+      <c r="C127" s="36">
+        <v>154.11726382556031</v>
+      </c>
+      <c r="D127" s="36">
+        <v>155.45452359364822</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="4">
+        <v>46204</v>
+      </c>
+      <c r="B128" s="17">
+        <v>151.55415093373639</v>
+      </c>
+      <c r="C128" s="36">
+        <v>149.64792298456885</v>
+      </c>
+      <c r="D128" s="36">
+        <v>155.76485474634373</v>
       </c>
     </row>
   </sheetData>
@@ -7677,14 +7689,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51" t="s">
+      <c r="C1" s="49"/>
+      <c r="D1" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="51"/>
+      <c r="E1" s="49"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -7705,16 +7717,16 @@
         <v>38</v>
       </c>
       <c r="B3">
-        <v>21</v>
+        <v>24.4</v>
       </c>
       <c r="C3">
-        <v>28.2</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="D3">
-        <v>4.8</v>
+        <v>5.6</v>
       </c>
       <c r="E3">
-        <v>6.3</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -7722,16 +7734,16 @@
         <v>39</v>
       </c>
       <c r="B4">
-        <v>7.3</v>
+        <v>8.9</v>
       </c>
       <c r="C4">
-        <v>9.6</v>
+        <v>11.1</v>
       </c>
       <c r="D4">
-        <v>2.2000000000000002</v>
+        <v>1.7</v>
       </c>
       <c r="E4">
-        <v>2.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -7739,16 +7751,16 @@
         <v>40</v>
       </c>
       <c r="B5">
-        <v>25.5</v>
+        <v>29.7</v>
       </c>
       <c r="C5">
-        <v>32.6</v>
+        <v>36.9</v>
       </c>
       <c r="D5">
-        <v>6.3</v>
+        <v>7.6</v>
       </c>
       <c r="E5">
-        <v>8</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -7756,16 +7768,16 @@
         <v>216</v>
       </c>
       <c r="B6">
-        <v>23.5</v>
+        <v>27.4</v>
       </c>
       <c r="C6">
-        <v>31.9</v>
+        <v>36.9</v>
       </c>
       <c r="D6">
-        <v>4.4000000000000004</v>
+        <v>5.4</v>
       </c>
       <c r="E6">
-        <v>5.5</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -7773,16 +7785,16 @@
         <v>217</v>
       </c>
       <c r="B7">
-        <v>25.5</v>
+        <v>27.4</v>
       </c>
       <c r="C7">
-        <v>34</v>
+        <v>36.799999999999997</v>
       </c>
       <c r="D7">
-        <v>2.9</v>
+        <v>1.4</v>
       </c>
       <c r="E7">
-        <v>3.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -7790,16 +7802,16 @@
         <v>41</v>
       </c>
       <c r="B8">
-        <v>23.2</v>
+        <v>26.9</v>
       </c>
       <c r="C8">
-        <v>30.1</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="D8">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="E8">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -7807,16 +7819,16 @@
         <v>42</v>
       </c>
       <c r="B9">
-        <v>23.5</v>
+        <v>29.5</v>
       </c>
       <c r="C9">
-        <v>31.3</v>
+        <v>41</v>
       </c>
       <c r="D9">
-        <v>5.6</v>
+        <v>6.9</v>
       </c>
       <c r="E9">
-        <v>7.6</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -7824,16 +7836,16 @@
         <v>43</v>
       </c>
       <c r="B10">
-        <v>19.7</v>
+        <v>24.4</v>
       </c>
       <c r="C10">
-        <v>27.9</v>
+        <v>29.9</v>
       </c>
       <c r="D10">
-        <v>2.7</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="E10">
-        <v>4.5999999999999996</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -7841,16 +7853,16 @@
         <v>218</v>
       </c>
       <c r="B11">
-        <v>34</v>
+        <v>40.299999999999997</v>
       </c>
       <c r="C11">
-        <v>42.2</v>
+        <v>48.6</v>
       </c>
       <c r="D11">
-        <v>10.6</v>
+        <v>14.2</v>
       </c>
       <c r="E11">
-        <v>13.2</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -7858,16 +7870,16 @@
         <v>44</v>
       </c>
       <c r="B12">
-        <v>22.2</v>
+        <v>30.2</v>
       </c>
       <c r="C12">
-        <v>27.3</v>
+        <v>42.2</v>
       </c>
       <c r="D12">
-        <v>2.9</v>
+        <v>6.3</v>
       </c>
       <c r="E12">
-        <v>3.2</v>
+        <v>8.1999999999999993</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -7875,16 +7887,16 @@
         <v>45</v>
       </c>
       <c r="B13">
-        <v>26.9</v>
+        <v>30.2</v>
       </c>
       <c r="C13" s="28">
-        <v>35.700000000000003</v>
+        <v>37.299999999999997</v>
       </c>
       <c r="D13">
-        <v>3.7</v>
+        <v>6.6</v>
       </c>
       <c r="E13">
-        <v>4.5999999999999996</v>
+        <v>8.3000000000000007</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -7892,16 +7904,16 @@
         <v>46</v>
       </c>
       <c r="B14">
-        <v>17.8</v>
+        <v>21.6</v>
       </c>
       <c r="C14">
-        <v>23.6</v>
+        <v>27.9</v>
       </c>
       <c r="D14">
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="E14">
-        <v>3.2</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -7909,16 +7921,16 @@
         <v>47</v>
       </c>
       <c r="B15">
-        <v>20.3</v>
+        <v>21.1</v>
       </c>
       <c r="C15">
-        <v>26.6</v>
+        <v>27.6</v>
       </c>
       <c r="D15">
-        <v>2.9</v>
+        <v>1.5</v>
       </c>
       <c r="E15">
-        <v>4</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -7926,16 +7938,16 @@
         <v>48</v>
       </c>
       <c r="B16">
-        <v>26.2</v>
+        <v>26.6</v>
       </c>
       <c r="C16">
-        <v>36.700000000000003</v>
+        <v>38.4</v>
       </c>
       <c r="D16">
-        <v>3.6</v>
+        <v>2.8</v>
       </c>
       <c r="E16">
-        <v>5.0999999999999996</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -7943,16 +7955,16 @@
         <v>49</v>
       </c>
       <c r="B17">
-        <v>22.5</v>
+        <v>22.9</v>
       </c>
       <c r="C17">
         <v>29.7</v>
       </c>
       <c r="D17">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="E17">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -7960,16 +7972,16 @@
         <v>219</v>
       </c>
       <c r="B18">
-        <v>20.6</v>
+        <v>25.6</v>
       </c>
       <c r="C18">
-        <v>29.4</v>
+        <v>38.5</v>
       </c>
       <c r="D18">
-        <v>2.2999999999999998</v>
+        <v>2.7</v>
       </c>
       <c r="E18">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -7977,16 +7989,16 @@
         <v>50</v>
       </c>
       <c r="B19">
-        <v>15.4</v>
+        <v>20.5</v>
       </c>
       <c r="C19">
-        <v>22.6</v>
+        <v>26.6</v>
       </c>
       <c r="D19">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="E19">
-        <v>7.1</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -7994,16 +8006,16 @@
         <v>220</v>
       </c>
       <c r="B20">
-        <v>39.299999999999997</v>
+        <v>43.6</v>
       </c>
       <c r="C20">
-        <v>49.9</v>
+        <v>56.2</v>
       </c>
       <c r="D20">
-        <v>9.8000000000000007</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="E20">
-        <v>13.6</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -8011,16 +8023,16 @@
         <v>51</v>
       </c>
       <c r="B21">
-        <v>16.8</v>
+        <v>21.3</v>
       </c>
       <c r="C21">
-        <v>23.2</v>
+        <v>31.1</v>
       </c>
       <c r="D21">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="E21">
-        <v>4.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -8028,16 +8040,16 @@
         <v>52</v>
       </c>
       <c r="B22">
-        <v>23.6</v>
+        <v>28</v>
       </c>
       <c r="C22">
-        <v>31.5</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="D22">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="E22">
-        <v>9</v>
+        <v>9.1999999999999993</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -8045,16 +8057,16 @@
         <v>53</v>
       </c>
       <c r="B23">
-        <v>16.600000000000001</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="C23">
-        <v>22.3</v>
+        <v>23.1</v>
       </c>
       <c r="D23">
-        <v>3.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="E23">
-        <v>3.9</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -8062,16 +8074,16 @@
         <v>221</v>
       </c>
       <c r="B24">
-        <v>21.7</v>
+        <v>25.1</v>
       </c>
       <c r="C24">
-        <v>31.1</v>
+        <v>34.299999999999997</v>
       </c>
       <c r="D24">
-        <v>6.2</v>
+        <v>4.7</v>
       </c>
       <c r="E24">
-        <v>8.8000000000000007</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -8079,16 +8091,16 @@
         <v>54</v>
       </c>
       <c r="B25">
-        <v>22.8</v>
+        <v>29</v>
       </c>
       <c r="C25">
-        <v>30.6</v>
+        <v>38.6</v>
       </c>
       <c r="D25">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="E25">
-        <v>9.3000000000000007</v>
+        <v>9.8000000000000007</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -8096,16 +8108,16 @@
         <v>55</v>
       </c>
       <c r="B26">
-        <v>17.899999999999999</v>
+        <v>14.9</v>
       </c>
       <c r="C26">
-        <v>22.8</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="D26">
         <v>4.3</v>
       </c>
       <c r="E26">
-        <v>5.2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -8113,16 +8125,16 @@
         <v>56</v>
       </c>
       <c r="B27">
-        <v>17.2</v>
+        <v>16.2</v>
       </c>
       <c r="C27">
-        <v>22.8</v>
+        <v>23.6</v>
       </c>
       <c r="D27">
-        <v>3.1</v>
+        <v>2.4</v>
       </c>
       <c r="E27">
-        <v>3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -8130,16 +8142,16 @@
         <v>57</v>
       </c>
       <c r="B28">
-        <v>17.2</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="C28">
-        <v>25.6</v>
+        <v>25.4</v>
       </c>
       <c r="D28">
-        <v>5.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="E28">
-        <v>8.6999999999999993</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -8147,16 +8159,16 @@
         <v>222</v>
       </c>
       <c r="B29">
-        <v>25</v>
+        <v>24.7</v>
       </c>
       <c r="C29">
-        <v>33.799999999999997</v>
+        <v>35.5</v>
       </c>
       <c r="D29">
-        <v>6.6</v>
+        <v>7</v>
       </c>
       <c r="E29">
-        <v>8.9</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -8164,16 +8176,16 @@
         <v>58</v>
       </c>
       <c r="B30">
-        <v>19</v>
+        <v>25.4</v>
       </c>
       <c r="C30">
-        <v>27.1</v>
+        <v>37.200000000000003</v>
       </c>
       <c r="D30">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="E30">
-        <v>4.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -8181,16 +8193,16 @@
         <v>223</v>
       </c>
       <c r="B31">
-        <v>18.3</v>
+        <v>15.7</v>
       </c>
       <c r="C31">
-        <v>22.4</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="D31">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E31">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -8198,16 +8210,16 @@
         <v>59</v>
       </c>
       <c r="B32">
-        <v>16.5</v>
+        <v>19.3</v>
       </c>
       <c r="C32">
-        <v>23.6</v>
+        <v>25.6</v>
       </c>
       <c r="D32">
-        <v>4.4000000000000004</v>
+        <v>1.8</v>
       </c>
       <c r="E32">
-        <v>4.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -8215,16 +8227,16 @@
         <v>60</v>
       </c>
       <c r="B33">
-        <v>16.2</v>
+        <v>19.5</v>
       </c>
       <c r="C33">
-        <v>22.6</v>
+        <v>25.9</v>
       </c>
       <c r="D33">
-        <v>3.4</v>
+        <v>2.6</v>
       </c>
       <c r="E33">
-        <v>4.3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -8232,16 +8244,16 @@
         <v>224</v>
       </c>
       <c r="B34">
-        <v>25.4</v>
+        <v>26.9</v>
       </c>
       <c r="C34">
-        <v>32.9</v>
+        <v>35.1</v>
       </c>
       <c r="D34">
-        <v>4.0999999999999996</v>
+        <v>8</v>
       </c>
       <c r="E34">
-        <v>5.9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -8249,16 +8261,16 @@
         <v>61</v>
       </c>
       <c r="B35">
-        <v>19.8</v>
+        <v>23.6</v>
       </c>
       <c r="C35">
-        <v>26.5</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="D35">
-        <v>2</v>
+        <v>3.8</v>
       </c>
       <c r="E35">
-        <v>3.2</v>
+        <v>5.2</v>
       </c>
     </row>
   </sheetData>
@@ -8283,14 +8295,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51" t="s">
+      <c r="C1" s="49"/>
+      <c r="D1" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="51"/>
+      <c r="E1" s="49"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8311,16 +8323,16 @@
         <v>62</v>
       </c>
       <c r="B3">
-        <v>21</v>
+        <v>24.4</v>
       </c>
       <c r="C3">
-        <v>28.2</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="D3">
-        <v>4.8</v>
+        <v>5.6</v>
       </c>
       <c r="E3">
-        <v>6.3</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -8328,16 +8340,16 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>24</v>
+        <v>24.9</v>
       </c>
       <c r="C4">
-        <v>32.299999999999997</v>
+        <v>32.1</v>
       </c>
       <c r="D4">
-        <v>3.7</v>
+        <v>6.2</v>
       </c>
       <c r="E4">
-        <v>4.5999999999999996</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -8345,16 +8357,16 @@
         <v>63</v>
       </c>
       <c r="B5">
-        <v>21.2</v>
+        <v>27.3</v>
       </c>
       <c r="C5">
-        <v>28.3</v>
+        <v>36.700000000000003</v>
       </c>
       <c r="D5">
-        <v>5.4</v>
+        <v>4</v>
       </c>
       <c r="E5">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -8362,16 +8374,16 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>25.5</v>
+        <v>31.9</v>
       </c>
       <c r="C6">
-        <v>32.700000000000003</v>
+        <v>41.5</v>
       </c>
       <c r="D6">
-        <v>5.8</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="E6">
-        <v>7.5</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -8379,16 +8391,16 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>21.1</v>
+        <v>23.6</v>
       </c>
       <c r="C7">
-        <v>28.4</v>
+        <v>31.5</v>
       </c>
       <c r="D7">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="E7">
-        <v>3.8</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -8396,16 +8408,16 @@
         <v>64</v>
       </c>
       <c r="B8">
-        <v>19.3</v>
+        <v>21.9</v>
       </c>
       <c r="C8">
-        <v>26.2</v>
+        <v>30.3</v>
       </c>
       <c r="D8">
-        <v>4.7</v>
+        <v>5.2</v>
       </c>
       <c r="E8">
-        <v>6.2</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -8413,16 +8425,16 @@
         <v>65</v>
       </c>
       <c r="B9">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C9">
-        <v>25.4</v>
+        <v>28.4</v>
       </c>
       <c r="D9">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E9">
-        <v>4</v>
+        <v>4.2</v>
       </c>
     </row>
   </sheetData>
@@ -8461,10 +8473,10 @@
       <c r="A2" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="46">
+      <c r="B2" s="44">
         <v>11730.33175329</v>
       </c>
-      <c r="C2" s="46">
+      <c r="C2" s="44">
         <v>14332.557392840001</v>
       </c>
       <c r="D2" s="27">
@@ -8476,10 +8488,10 @@
       <c r="A3" s="32" t="s">
         <v>203</v>
       </c>
-      <c r="B3" s="42">
+      <c r="B3" s="40">
         <v>8577.9098430699996</v>
       </c>
-      <c r="C3" s="42">
+      <c r="C3" s="40">
         <v>10629.94907769</v>
       </c>
       <c r="D3" s="27">
@@ -8491,10 +8503,10 @@
       <c r="A4" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="B4" s="42">
+      <c r="B4" s="40">
         <v>1199.62775519</v>
       </c>
-      <c r="C4" s="42">
+      <c r="C4" s="40">
         <v>3296.06363272</v>
       </c>
       <c r="D4" s="27">
@@ -8506,10 +8518,10 @@
       <c r="A5" s="32" t="s">
         <v>209</v>
       </c>
-      <c r="B5" s="42">
+      <c r="B5" s="40">
         <v>1505.5014949900001</v>
       </c>
-      <c r="C5" s="42">
+      <c r="C5" s="40">
         <v>400.64444258999998</v>
       </c>
       <c r="D5" s="27">
@@ -8521,10 +8533,10 @@
       <c r="A6" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="46">
+      <c r="B6" s="44">
         <v>8316.7128498999991</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="44">
         <v>1561.26989688</v>
       </c>
       <c r="D6" s="27">
@@ -8536,10 +8548,10 @@
       <c r="A7" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="42">
+      <c r="B7" s="40">
         <v>4288.9319074699997</v>
       </c>
-      <c r="C7" s="42">
+      <c r="C7" s="40">
         <v>575.48966665</v>
       </c>
       <c r="D7" s="27">
@@ -8551,10 +8563,10 @@
       <c r="A8" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="B8" s="42">
+      <c r="B8" s="40">
         <v>2002.80556398</v>
       </c>
-      <c r="C8" s="42">
+      <c r="C8" s="40">
         <v>200.23070425</v>
       </c>
       <c r="D8" s="27">
@@ -8566,10 +8578,10 @@
       <c r="A9" s="31" t="s">
         <v>175</v>
       </c>
-      <c r="B9" s="46">
+      <c r="B9" s="44">
         <v>8171.8416171899999</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="44">
         <v>5900.1284501500004</v>
       </c>
       <c r="D9" s="27">
@@ -8581,10 +8593,10 @@
       <c r="A10" s="32" t="s">
         <v>205</v>
       </c>
-      <c r="B10" s="42">
+      <c r="B10" s="40">
         <v>6691.4666677699997</v>
       </c>
-      <c r="C10" s="42">
+      <c r="C10" s="40">
         <v>4529.8080052300002</v>
       </c>
       <c r="D10" s="27">
@@ -8596,10 +8608,10 @@
       <c r="A11" s="31" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="46">
+      <c r="B11" s="44">
         <v>6222.0785865199996</v>
       </c>
-      <c r="C11" s="46">
+      <c r="C11" s="44">
         <v>6625.6950472400003</v>
       </c>
       <c r="D11" s="27">
@@ -8611,10 +8623,10 @@
       <c r="A12" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="B12" s="42">
+      <c r="B12" s="40">
         <v>769.16592227000001</v>
       </c>
-      <c r="C12" s="42">
+      <c r="C12" s="40">
         <v>2053.1686061700002</v>
       </c>
       <c r="D12" s="27">
@@ -8626,10 +8638,10 @@
       <c r="A13" s="32" t="s">
         <v>213</v>
       </c>
-      <c r="B13" s="42">
+      <c r="B13" s="40">
         <v>1128.9283964700001</v>
       </c>
-      <c r="C13" s="42">
+      <c r="C13" s="40">
         <v>687.46461611999996</v>
       </c>
       <c r="D13" s="27">
@@ -8641,10 +8653,10 @@
       <c r="A14" s="32" t="s">
         <v>214</v>
       </c>
-      <c r="B14" s="42">
+      <c r="B14" s="40">
         <v>770.90505522000001</v>
       </c>
-      <c r="C14" s="42">
+      <c r="C14" s="40">
         <v>1025.9636580599999</v>
       </c>
       <c r="D14" s="27">
@@ -8656,10 +8668,10 @@
       <c r="A15" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="B15" s="42">
+      <c r="B15" s="40">
         <v>1356.0770490699999</v>
       </c>
-      <c r="C15" s="42">
+      <c r="C15" s="40">
         <v>215.60331056999999</v>
       </c>
       <c r="D15" s="27">
@@ -8671,10 +8683,10 @@
       <c r="A16" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="46">
+      <c r="B16" s="44">
         <v>6155.1991863900002</v>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="44">
         <v>11229.9276689</v>
       </c>
       <c r="D16" s="27">
@@ -8686,10 +8698,10 @@
       <c r="A17" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="46">
+      <c r="B17" s="44">
         <v>4276.45312431</v>
       </c>
-      <c r="C17" s="46">
+      <c r="C17" s="44">
         <v>779.18460789999995</v>
       </c>
       <c r="D17" s="27">
@@ -8701,10 +8713,10 @@
       <c r="A18" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="B18" s="46">
+      <c r="B18" s="44">
         <v>6316.4825914599996</v>
       </c>
-      <c r="C18" s="46">
+      <c r="C18" s="44">
         <v>2661.3959148200001</v>
       </c>
       <c r="D18" s="27">
@@ -8716,10 +8728,10 @@
       <c r="A19" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="B19" s="42">
+      <c r="B19" s="40">
         <v>1035.20953153</v>
       </c>
-      <c r="C19" s="42">
+      <c r="C19" s="40">
         <v>287.44898253000002</v>
       </c>
       <c r="D19" s="27">
@@ -8731,10 +8743,10 @@
       <c r="A20" s="32" t="s">
         <v>210</v>
       </c>
-      <c r="B20" s="42">
+      <c r="B20" s="40">
         <v>1170.8101533199999</v>
       </c>
-      <c r="C20" s="42">
+      <c r="C20" s="40">
         <v>151.96947852</v>
       </c>
       <c r="D20" s="27">
@@ -8746,10 +8758,10 @@
       <c r="A21" s="32" t="s">
         <v>211</v>
       </c>
-      <c r="B21" s="42">
+      <c r="B21" s="40">
         <v>1136.0953787399999</v>
       </c>
-      <c r="C21" s="42">
+      <c r="C21" s="40">
         <v>1349.22044682</v>
       </c>
       <c r="D21" s="27">
@@ -8761,10 +8773,10 @@
       <c r="A22" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="B22" s="42">
+      <c r="B22" s="40">
         <v>2421.13608991</v>
       </c>
-      <c r="C22" s="42">
+      <c r="C22" s="40">
         <v>669.25282884000001</v>
       </c>
       <c r="D22" s="27">
@@ -8776,10 +8788,10 @@
       <c r="A23" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="46">
+      <c r="B23" s="44">
         <v>3400.7110296199999</v>
       </c>
-      <c r="C23" s="46">
+      <c r="C23" s="44">
         <v>325.37604098000003</v>
       </c>
       <c r="D23" s="27">
@@ -8791,10 +8803,10 @@
       <c r="A24" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="46">
+      <c r="B24" s="44">
         <v>2723.3428194799999</v>
       </c>
-      <c r="C24" s="46">
+      <c r="C24" s="44">
         <v>427.87939122</v>
       </c>
       <c r="D24" s="27">
@@ -8806,10 +8818,10 @@
       <c r="A25" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="B25" s="46">
+      <c r="B25" s="44">
         <v>229.78354913999999</v>
       </c>
-      <c r="C25" s="46">
+      <c r="C25" s="44">
         <v>136.89460957</v>
       </c>
       <c r="D25" s="27">
@@ -8821,10 +8833,10 @@
       <c r="A26" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B26" s="46">
+      <c r="B26" s="44">
         <v>755.64002840000001</v>
       </c>
-      <c r="C26" s="46">
+      <c r="C26" s="44">
         <v>226.26251718</v>
       </c>
       <c r="D26" s="27">
@@ -8836,10 +8848,10 @@
       <c r="A27" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="47">
+      <c r="B27" s="45">
         <v>8949.1916499800009</v>
       </c>
-      <c r="C27" s="47">
+      <c r="C27" s="45">
         <v>4792.11866758</v>
       </c>
       <c r="D27" s="27">
@@ -8873,7 +8885,7 @@
       <c r="A2" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="48">
+      <c r="B2" s="46">
         <v>67247.768785680004</v>
       </c>
       <c r="D2" s="29"/>
@@ -8882,7 +8894,7 @@
       <c r="A3" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="B3" s="48">
+      <c r="B3" s="46">
         <v>16480.22902545</v>
       </c>
       <c r="D3" s="29"/>
@@ -8891,7 +8903,7 @@
       <c r="A4" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="49">
+      <c r="B4" s="47">
         <v>20.101308509999999</v>
       </c>
       <c r="D4" s="30"/>
@@ -8900,7 +8912,7 @@
       <c r="A5" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="49">
+      <c r="B5" s="47">
         <v>1468.3693771000001</v>
       </c>
       <c r="D5" s="30"/>
@@ -8909,7 +8921,7 @@
       <c r="A6" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="49">
+      <c r="B6" s="47">
         <v>223.15063314</v>
       </c>
       <c r="D6" s="30"/>
@@ -8918,7 +8930,7 @@
       <c r="A7" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="49">
+      <c r="B7" s="47">
         <v>535.44731380999997</v>
       </c>
       <c r="D7" s="30"/>
@@ -8927,7 +8939,7 @@
       <c r="A8" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="B8" s="49">
+      <c r="B8" s="47">
         <v>561.20805385000006</v>
       </c>
       <c r="D8" s="30"/>
@@ -8936,7 +8948,7 @@
       <c r="A9" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B9" s="49">
+      <c r="B9" s="47">
         <v>9772.09621591</v>
       </c>
       <c r="D9" s="30"/>
@@ -8945,7 +8957,7 @@
       <c r="A10" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="49">
+      <c r="B10" s="47">
         <v>2662.54073986</v>
       </c>
       <c r="D10" s="30"/>
@@ -8954,7 +8966,7 @@
       <c r="A11" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="B11" s="49">
+      <c r="B11" s="47">
         <v>190.99193421000001</v>
       </c>
       <c r="D11" s="30"/>
@@ -8963,7 +8975,7 @@
       <c r="A12" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="B12" s="49">
+      <c r="B12" s="47">
         <v>70.052651049999994</v>
       </c>
       <c r="D12" s="30"/>
@@ -8972,7 +8984,7 @@
       <c r="A13" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="B13" s="49">
+      <c r="B13" s="47">
         <v>87.533367830000003</v>
       </c>
       <c r="D13" s="30"/>
@@ -8981,7 +8993,7 @@
       <c r="A14" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B14" s="49">
+      <c r="B14" s="47">
         <v>748.84156416999997</v>
       </c>
       <c r="D14" s="30"/>
@@ -8990,7 +9002,7 @@
       <c r="A15" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="49">
+      <c r="B15" s="47">
         <v>139.89586600999999</v>
       </c>
       <c r="D15" s="30"/>
@@ -8999,7 +9011,7 @@
       <c r="A16" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="B16" s="48">
+      <c r="B16" s="46">
         <v>22206.062888460001</v>
       </c>
       <c r="D16" s="29"/>
@@ -9008,7 +9020,7 @@
       <c r="A17" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="49">
+      <c r="B17" s="47">
         <v>3670.0701619699998</v>
       </c>
       <c r="D17" s="30"/>
@@ -9017,7 +9029,7 @@
       <c r="A18" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="B18" s="49">
+      <c r="B18" s="47">
         <v>208.18073641000001</v>
       </c>
       <c r="D18" s="30"/>
@@ -9026,7 +9038,7 @@
       <c r="A19" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="B19" s="49">
+      <c r="B19" s="47">
         <v>977.86101798000004</v>
       </c>
       <c r="D19" s="30"/>
@@ -9035,7 +9047,7 @@
       <c r="A20" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="B20" s="49">
+      <c r="B20" s="47">
         <v>67.576166659999998</v>
       </c>
       <c r="D20" s="30"/>
@@ -9044,7 +9056,7 @@
       <c r="A21" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="B21" s="49">
+      <c r="B21" s="47">
         <v>81.563704099999995</v>
       </c>
       <c r="D21" s="30"/>
@@ -9053,7 +9065,7 @@
       <c r="A22" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="49">
+      <c r="B22" s="47">
         <v>127.5469717</v>
       </c>
       <c r="D22" s="30"/>
@@ -9062,7 +9074,7 @@
       <c r="A23" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="B23" s="49">
+      <c r="B23" s="47">
         <v>527.70245546000001</v>
       </c>
       <c r="D23" s="30"/>
@@ -9071,7 +9083,7 @@
       <c r="A24" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="B24" s="49">
+      <c r="B24" s="47">
         <v>7391.6640766999999</v>
       </c>
       <c r="D24" s="30"/>
@@ -9080,7 +9092,7 @@
       <c r="A25" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B25" s="49">
+      <c r="B25" s="47">
         <v>253.92114058000001</v>
       </c>
       <c r="D25" s="30"/>
@@ -9089,7 +9101,7 @@
       <c r="A26" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="B26" s="49">
+      <c r="B26" s="47">
         <v>722.88290491999999</v>
       </c>
       <c r="D26" s="30"/>
@@ -9098,7 +9110,7 @@
       <c r="A27" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="B27" s="49">
+      <c r="B27" s="47">
         <v>478.13456760000003</v>
       </c>
       <c r="D27" s="30"/>
@@ -9107,7 +9119,7 @@
       <c r="A28" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="B28" s="49">
+      <c r="B28" s="47">
         <v>6685.94059664</v>
       </c>
       <c r="D28" s="30"/>
@@ -9116,7 +9128,7 @@
       <c r="A29" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="B29" s="49">
+      <c r="B29" s="47">
         <v>212.31669382999999</v>
       </c>
       <c r="D29" s="30"/>
@@ -9125,7 +9137,7 @@
       <c r="A30" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="B30" s="49">
+      <c r="B30" s="47">
         <v>238.07436966</v>
       </c>
       <c r="D30" s="30"/>
@@ -9134,7 +9146,7 @@
       <c r="A31" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="B31" s="49">
+      <c r="B31" s="47">
         <v>91.66533622</v>
       </c>
       <c r="D31" s="30"/>
@@ -9143,7 +9155,7 @@
       <c r="A32" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="B32" s="49">
+      <c r="B32" s="47">
         <v>470.96198802999999</v>
       </c>
       <c r="D32" s="30"/>
@@ -9152,7 +9164,7 @@
       <c r="A33" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="B33" s="48">
+      <c r="B33" s="46">
         <v>17894.47491017</v>
       </c>
       <c r="D33" s="29"/>
@@ -9161,7 +9173,7 @@
       <c r="A34" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="B34" s="49">
+      <c r="B34" s="47">
         <v>4152.2687079099996</v>
       </c>
       <c r="D34" s="30"/>
@@ -9170,7 +9182,7 @@
       <c r="A35" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="B35" s="49">
+      <c r="B35" s="47">
         <v>822.11696787999995</v>
       </c>
       <c r="D35" s="30"/>
@@ -9179,7 +9191,7 @@
       <c r="A36" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="B36" s="49">
+      <c r="B36" s="47">
         <v>115.9260226</v>
       </c>
       <c r="D36" s="30"/>
@@ -9188,7 +9200,7 @@
       <c r="A37" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="B37" s="49">
+      <c r="B37" s="47">
         <v>11.98579423</v>
       </c>
       <c r="D37" s="30"/>
@@ -9197,7 +9209,7 @@
       <c r="A38" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="B38" s="49">
+      <c r="B38" s="47">
         <v>268.75686449</v>
       </c>
       <c r="D38" s="30"/>
@@ -9206,7 +9218,7 @@
       <c r="A39" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="B39" s="49">
+      <c r="B39" s="47">
         <v>69.535566700000004</v>
       </c>
       <c r="D39" s="30"/>
@@ -9215,7 +9227,7 @@
       <c r="A40" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="B40" s="49">
+      <c r="B40" s="47">
         <v>5.6628988700000003</v>
       </c>
       <c r="D40" s="30"/>
@@ -9224,7 +9236,7 @@
       <c r="A41" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="49">
+      <c r="B41" s="47">
         <v>86.869893590000004</v>
       </c>
       <c r="D41" s="30"/>
@@ -9233,7 +9245,7 @@
       <c r="A42" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="B42" s="49">
+      <c r="B42" s="47">
         <v>3669.6649587400002</v>
       </c>
       <c r="D42" s="30"/>
@@ -9242,7 +9254,7 @@
       <c r="A43" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B43" s="49">
+      <c r="B43" s="47">
         <v>1824.52611748</v>
       </c>
       <c r="D43" s="30"/>
@@ -9251,7 +9263,7 @@
       <c r="A44" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="B44" s="49">
+      <c r="B44" s="47">
         <v>905.29051629000003</v>
       </c>
       <c r="D44" s="30"/>
@@ -9260,7 +9272,7 @@
       <c r="A45" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="B45" s="49">
+      <c r="B45" s="47">
         <v>5443.3517914000004</v>
       </c>
       <c r="D45" s="30"/>
@@ -9269,7 +9281,7 @@
       <c r="A46" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B46" s="49">
+      <c r="B46" s="47">
         <v>108.64312488</v>
       </c>
       <c r="D46" s="30"/>
@@ -9278,7 +9290,7 @@
       <c r="A47" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="B47" s="49">
+      <c r="B47" s="47">
         <v>409.87568511000001</v>
       </c>
       <c r="D47" s="30"/>
@@ -9287,7 +9299,7 @@
       <c r="A48" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="B48" s="48">
+      <c r="B48" s="46">
         <v>10667.001961600001</v>
       </c>
       <c r="D48" s="29"/>
@@ -9296,7 +9308,7 @@
       <c r="A49" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B49" s="49">
+      <c r="B49" s="47">
         <v>6625.3174199499999</v>
       </c>
       <c r="D49" s="30"/>
@@ -9305,7 +9317,7 @@
       <c r="A50" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="B50" s="49">
+      <c r="B50" s="47">
         <v>2563.0320099300002</v>
       </c>
       <c r="D50" s="30"/>
@@ -9314,7 +9326,7 @@
       <c r="A51" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="B51" s="49">
+      <c r="B51" s="47">
         <v>83.760430099999994</v>
       </c>
       <c r="D51" s="30"/>
@@ -9323,7 +9335,7 @@
       <c r="A52" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="B52" s="42">
+      <c r="B52" s="40">
         <v>1040.1389722199999</v>
       </c>
       <c r="D52" s="30"/>
@@ -9332,7 +9344,7 @@
       <c r="A53" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="B53" s="50">
+      <c r="B53" s="48">
         <v>354.75312939999998</v>
       </c>
     </row>
@@ -9362,7 +9374,7 @@
       <c r="A2" s="33" t="s">
         <v>177</v>
       </c>
-      <c r="B2" s="43">
+      <c r="B2" s="41">
         <v>48998.690205259998</v>
       </c>
     </row>
@@ -9370,7 +9382,7 @@
       <c r="A3" s="33" t="s">
         <v>178</v>
       </c>
-      <c r="B3" s="43">
+      <c r="B3" s="41">
         <v>9276.8012137000005</v>
       </c>
     </row>
@@ -9378,7 +9390,7 @@
       <c r="A4" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="B4" s="44">
+      <c r="B4" s="42">
         <v>1043.99740019</v>
       </c>
     </row>
@@ -9386,7 +9398,7 @@
       <c r="A5" s="34" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="44">
+      <c r="B5" s="42">
         <v>1603.6225589400001</v>
       </c>
     </row>
@@ -9394,7 +9406,7 @@
       <c r="A6" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="B6" s="44">
+      <c r="B6" s="42">
         <v>16949.051997629998</v>
       </c>
     </row>
@@ -9402,7 +9414,7 @@
       <c r="A7" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="B7" s="43">
+      <c r="B7" s="41">
         <v>2932.0284670599999</v>
       </c>
     </row>
@@ -9410,7 +9422,7 @@
       <c r="A8" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="B8" s="44">
+      <c r="B8" s="42">
         <v>410.84743400999997</v>
       </c>
     </row>
@@ -9418,7 +9430,7 @@
       <c r="A9" s="34" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="44">
+      <c r="B9" s="42">
         <v>655.31856334999998</v>
       </c>
     </row>
@@ -9426,7 +9438,7 @@
       <c r="A10" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="44">
+      <c r="B10" s="42">
         <v>11583.69053021</v>
       </c>
     </row>
@@ -9434,7 +9446,7 @@
       <c r="A11" s="34" t="s">
         <v>186</v>
       </c>
-      <c r="B11" s="44">
+      <c r="B11" s="42">
         <v>1367.167003</v>
       </c>
     </row>
@@ -9442,7 +9454,7 @@
       <c r="A12" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="B12" s="44">
+      <c r="B12" s="42">
         <v>2832.5070699500002</v>
       </c>
     </row>
@@ -9450,7 +9462,7 @@
       <c r="A13" s="33" t="s">
         <v>188</v>
       </c>
-      <c r="B13" s="43">
+      <c r="B13" s="41">
         <v>297.24078580000003</v>
       </c>
     </row>
@@ -9458,7 +9470,7 @@
       <c r="A14" s="34" t="s">
         <v>189</v>
       </c>
-      <c r="B14" s="44">
+      <c r="B14" s="42">
         <v>2535.26628415</v>
       </c>
     </row>
@@ -9466,7 +9478,7 @@
       <c r="A15" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="B15" s="44">
+      <c r="B15" s="42">
         <v>8386.5318090199999</v>
       </c>
     </row>
@@ -9474,7 +9486,7 @@
       <c r="A16" s="33" t="s">
         <v>191</v>
       </c>
-      <c r="B16" s="43">
+      <c r="B16" s="41">
         <v>3215.9855721600002</v>
       </c>
     </row>
@@ -9482,7 +9494,7 @@
       <c r="A17" s="34" t="s">
         <v>192</v>
       </c>
-      <c r="B17" s="44">
+      <c r="B17" s="42">
         <v>445.37679042000002</v>
       </c>
     </row>
@@ -9490,7 +9502,7 @@
       <c r="A18" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="B18" s="44">
+      <c r="B18" s="42">
         <v>4725.1694464399998</v>
       </c>
     </row>
@@ -9498,7 +9510,7 @@
       <c r="A19" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="B19" s="44">
+      <c r="B19" s="42">
         <v>7192.7584739699996</v>
       </c>
     </row>
@@ -9506,7 +9518,7 @@
       <c r="A20" s="33" t="s">
         <v>195</v>
       </c>
-      <c r="B20" s="43">
+      <c r="B20" s="41">
         <v>555.51545514999998</v>
       </c>
     </row>
@@ -9514,7 +9526,7 @@
       <c r="A21" s="34" t="s">
         <v>196</v>
       </c>
-      <c r="B21" s="44">
+      <c r="B21" s="42">
         <v>1067.8667938200001</v>
       </c>
     </row>
@@ -9522,7 +9534,7 @@
       <c r="A22" s="34" t="s">
         <v>197</v>
       </c>
-      <c r="B22" s="44">
+      <c r="B22" s="42">
         <v>6629.1812545700004</v>
       </c>
     </row>
@@ -9530,7 +9542,7 @@
       <c r="A23" s="34" t="s">
         <v>198</v>
       </c>
-      <c r="B23" s="44">
+      <c r="B23" s="42">
         <v>588.55855565000002</v>
       </c>
     </row>
@@ -9538,7 +9550,7 @@
       <c r="A24" s="34" t="s">
         <v>199</v>
       </c>
-      <c r="B24" s="44">
+      <c r="B24" s="42">
         <v>757.31480059</v>
       </c>
     </row>
@@ -9546,7 +9558,7 @@
       <c r="A25" s="34" t="s">
         <v>200</v>
       </c>
-      <c r="B25" s="44">
+      <c r="B25" s="42">
         <v>1860.5448149700001</v>
       </c>
     </row>
@@ -9554,7 +9566,7 @@
       <c r="A26" s="34" t="s">
         <v>201</v>
       </c>
-      <c r="B26" s="44">
+      <c r="B26" s="42">
         <v>1326.24926863</v>
       </c>
     </row>
@@ -9562,7 +9574,7 @@
       <c r="A27" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="B27" s="44">
+      <c r="B27" s="42">
         <v>1036.7040162799999</v>
       </c>
     </row>
@@ -9570,7 +9582,7 @@
       <c r="A28" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="B28" s="44">
+      <c r="B28" s="42">
         <v>3468.9390560100001</v>
       </c>
     </row>
@@ -9578,12 +9590,12 @@
       <c r="A29" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="B29" s="43">
+      <c r="B29" s="41">
         <v>892.10058498000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B30" s="45">
+      <c r="B30" s="43">
         <v>782.94421930999999</v>
       </c>
     </row>

</xml_diff>